<commit_message>
feat: carrusel de la entrega en Temixco en Aulas Tecnologicas
- Modulo carrusel.js reutilizable (Inicio y Aulas).
- Seccion de la entrega en la Primaria Miguel Hidalgo (nota del
  12/04/2026) con 4 fotos, cifras de la escuela y boton al mapa.
- Cita de Aulas con barra dorada; borrador en nahuatl de textos nuevos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traducciones/Traduccion_nahuatl_tablero.xlsx
+++ b/traducciones/Traduccion_nahuatl_tablero.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$G$335</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$G$347</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G335"/>
+  <dimension ref="A1:G347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7872,12 +7872,12 @@
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>Acercar tecnología a las escuelas es abrir oportunidades reales para las niñas y los niños, especialmente en zonas donde el acceso ha sido limitado.</t>
+          <t>{n} de abril de {n} · {d}</t>
         </is>
       </c>
       <c r="E237" s="5" t="inlineStr">
         <is>
-          <t>Tikitkiliskej tepostlapoualli ipan kaltlamachtiloyan kiijtosneki tiktlapoaj melauak ojmej iga pipiltontij, ogachi kanin amo asiaya.</t>
+          <t>{n} abril, {n} xiuitl · {d}</t>
         </is>
       </c>
       <c r="F237" s="4" t="inlineStr">
@@ -7903,12 +7903,12 @@
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>, director de Agenda Digital de la ATDEM, durante una entrega en Jojutla.</t>
+          <t>Entrega en la Escuela {d}</t>
         </is>
       </c>
       <c r="E238" s="5" t="inlineStr">
         <is>
-          <t>, tlayekanki ipan Agenda Digital ATDEM, kuak kitemakak ipan Jojutla.</t>
+          <t>Temakalistle ipan Kaltlamachtiloyan {d}</t>
         </is>
       </c>
       <c r="F238" s="4" t="inlineStr">
@@ -7934,12 +7934,12 @@
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>Escuelas por nivel educativo</t>
+          <t>La ATDEM instaló computadoras con software educativo y conexión a internet en la Escuela {d}, en la colonia {d} de {d}, una escuela en zona de atención prioritaria.</t>
         </is>
       </c>
       <c r="E239" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan iga temachtilistle</t>
+          <t>ATDEM kitlalij tepostlapoualli iga programas iga temachtilistle uan internet ipan Kaltlamachtiloyan {d}, ipan colonia {d} ipan {d}, se kaltlamachtiloyan kanin achtopa moneki tlapaleuilistle.</t>
         </is>
       </c>
       <c r="F239" s="4" t="inlineStr">
@@ -7965,12 +7965,12 @@
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>¿Dónde están las aulas?</t>
+          <t>computadoras en el aula</t>
         </is>
       </c>
       <c r="E240" s="5" t="inlineStr">
         <is>
-          <t>¿Kanin katej tlamachtiloyan?</t>
+          <t>tepostlapoualli ipan tlamachtiloyan</t>
         </is>
       </c>
       <c r="F240" s="4" t="inlineStr">
@@ -7996,12 +7996,12 @@
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>Todos los municipios</t>
+          <t>nivel educativo</t>
         </is>
       </c>
       <c r="E241" s="5" t="inlineStr">
         <is>
-          <t>Nochi altepemej</t>
+          <t>itemachtilis</t>
         </is>
       </c>
       <c r="F241" s="4" t="inlineStr">
@@ -8027,12 +8027,12 @@
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>Escuelas equipadas</t>
+          <t>“La transformación digital en Morelos tiene un propósito claro: que ninguna niña o niño se quede atrás.”</t>
         </is>
       </c>
       <c r="E242" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan tlen kipiaj tepostlapoualli</t>
+          <t>“Tlapatlalistle iga tepostlapoualli ipan Morelos kipia se melauak tlen guinegui: ma amigaj ichpogakonetl o piltontle mokaua iteipan.”</t>
         </is>
       </c>
       <c r="F242" s="4" t="inlineStr">
@@ -8058,12 +8058,12 @@
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t>Computadoras</t>
+          <t>Daniel Sotelo Salazar, director de Agenda Digital de la ATDEM</t>
         </is>
       </c>
       <c r="E243" s="5" t="inlineStr">
         <is>
-          <t>Tepostlapoualmej</t>
+          <t>Daniel Sotelo Salazar, tlayekanki ipan Agenda Digital ATDEM</t>
         </is>
       </c>
       <c r="F243" s="4" t="inlineStr">
@@ -8084,17 +8084,17 @@
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>Escuelas dentro de un polígono</t>
+          <t>Fotos de la entrega en {d}</t>
         </is>
       </c>
       <c r="E244" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan ipan se polígono</t>
+          <t>Ixkopinkayomej tlen temakalistle ipan {d}</t>
         </is>
       </c>
       <c r="F244" s="4" t="inlineStr">
@@ -8115,17 +8115,17 @@
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>Mapa de Aulas</t>
+          <t>Inauguración del aula de cómputo en la Escuela {d}, {d}.</t>
         </is>
       </c>
       <c r="E245" s="5" t="inlineStr">
         <is>
-          <t>Tlalamatl iga tlamachtiloyan</t>
+          <t>Peualistle tlen tlamachtiloyan iga tepostlapoualli ipan Kaltlamachtiloyan {d}, {d}.</t>
         </is>
       </c>
       <c r="F245" s="4" t="inlineStr">
@@ -8146,17 +8146,17 @@
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>El tamaño del círculo indica el número de computadoras. Haz clic en una escuela para ver su detalle.</t>
+          <t>Aula equipada con computadoras, software educativo y conexión a internet.</t>
         </is>
       </c>
       <c r="E246" s="5" t="inlineStr">
         <is>
-          <t>Kenin ueyi yaualtik kinextia keski tepostlapoualli kipia. Xikpacho se kaltlamachtiloyan iga tikitas nochi.</t>
+          <t>Tlamachtiloyan iga tepostlapoualli, programas iga temachtilistle uan internet.</t>
         </is>
       </c>
       <c r="F246" s="4" t="inlineStr">
@@ -8177,17 +8177,17 @@
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>Computadoras por aula</t>
+          <t>Entrega del aula a la comunidad escolar.</t>
         </is>
       </c>
       <c r="E247" s="5" t="inlineStr">
         <is>
-          <t>Tepostlapoualli ipan nochi tlamachtiloyan</t>
+          <t>Kitemakakej tlamachtiloyan ipan tlatlaga tlen kaltlamachtiloyan.</t>
         </is>
       </c>
       <c r="F247" s="4" t="inlineStr">
@@ -8208,17 +8208,17 @@
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>Municipio con aula</t>
+          <t>Ceremonia de entrega en la colonia {d}.</t>
         </is>
       </c>
       <c r="E248" s="5" t="inlineStr">
         <is>
-          <t>Altepetl iga tlamachtiloyan</t>
+          <t>Temakalistle ipan colonia {d}.</t>
         </is>
       </c>
       <c r="F248" s="4" t="inlineStr">
@@ -8244,12 +8244,12 @@
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>Otros municipios</t>
+          <t>Acercar tecnología a las escuelas es abrir oportunidades reales para las niñas y los niños, especialmente en zonas donde el acceso ha sido limitado.</t>
         </is>
       </c>
       <c r="E249" s="5" t="inlineStr">
         <is>
-          <t>Siguin altepemej</t>
+          <t>Tikitkiliskej tepostlapoualli ipan kaltlamachtiloyan kiijtosneki tiktlapoaj melauak ojmej iga pipiltontij, ogachi kanin amo asiaya.</t>
         </is>
       </c>
       <c r="F249" s="4" t="inlineStr">
@@ -8275,12 +8275,12 @@
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>Equipos por Municipio</t>
+          <t>, director de Agenda Digital de la ATDEM, durante una entrega en Jojutla.</t>
         </is>
       </c>
       <c r="E250" s="5" t="inlineStr">
         <is>
-          <t>Tepostlapoualli iga altepetl</t>
+          <t>, tlayekanki ipan Agenda Digital ATDEM, kuak kitemakak ipan Jojutla.</t>
         </is>
       </c>
       <c r="F250" s="4" t="inlineStr">
@@ -8306,12 +8306,12 @@
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t>{n} eq. · {n} esc.</t>
+          <t>Escuelas por nivel educativo</t>
         </is>
       </c>
       <c r="E251" s="5" t="inlineStr">
         <is>
-          <t>{n} tep. · {n} kal.</t>
+          <t>Kaltlamachtiloyan iga temachtilistle</t>
         </is>
       </c>
       <c r="F251" s="4" t="inlineStr">
@@ -8337,12 +8337,12 @@
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>Escuelas</t>
+          <t>¿Dónde están las aulas?</t>
         </is>
       </c>
       <c r="E252" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan</t>
+          <t>¿Kanin katej tlamachtiloyan?</t>
         </is>
       </c>
       <c r="F252" s="4" t="inlineStr">
@@ -8368,12 +8368,12 @@
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t>Escuela</t>
+          <t>Todos los municipios</t>
         </is>
       </c>
       <c r="E253" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan</t>
+          <t>Nochi altepemej</t>
         </is>
       </c>
       <c r="F253" s="4" t="inlineStr">
@@ -8399,12 +8399,12 @@
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>Equipos</t>
+          <t>Escuelas equipadas</t>
         </is>
       </c>
       <c r="E254" s="5" t="inlineStr">
         <is>
-          <t>Tepostlapoualmej</t>
+          <t>Kaltlamachtiloyan tlen kipiaj tepostlapoualli</t>
         </is>
       </c>
       <c r="F254" s="4" t="inlineStr">
@@ -8425,17 +8425,17 @@
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>Ver {d} en el mapa</t>
+          <t>Computadoras</t>
         </is>
       </c>
       <c r="E255" s="5" t="inlineStr">
         <is>
-          <t>Xikita {d} ipan tlalamatl</t>
+          <t>Tepostlapoualmej</t>
         </is>
       </c>
       <c r="F255" s="4" t="inlineStr">
@@ -8461,12 +8461,12 @@
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, "Proyecto Escuelas entrega Computadoras" (hoja Concentrado). Ubicación según el enlace de Google Maps capturado por escuela.</t>
+          <t>Escuelas dentro de un polígono</t>
         </is>
       </c>
       <c r="E256" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, "Proyecto Escuelas entrega Computadoras" (hoja Concentrado). Kanin katej iga ojtle Google Maps tlen motlalij iga nochi kaltlamachtiloyan.</t>
+          <t>Kaltlamachtiloyan ipan se polígono</t>
         </is>
       </c>
       <c r="F256" s="4" t="inlineStr">
@@ -8482,7 +8482,7 @@
       </c>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C257" s="4" t="inlineStr">
@@ -8492,12 +8492,12 @@
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>Conectividad pública · Agencia de Transformación Digital</t>
+          <t>Mapa de Aulas</t>
         </is>
       </c>
       <c r="E257" s="5" t="inlineStr">
         <is>
-          <t>Matlatl tlapojtok · Agencia de Transformación Digital</t>
+          <t>Tlalamatl iga tlamachtiloyan</t>
         </is>
       </c>
       <c r="F257" s="4" t="inlineStr">
@@ -8513,7 +8513,7 @@
       </c>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr">
@@ -8523,12 +8523,12 @@
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t>Red de Wi-Fi pública, gratuita y abierta impulsada por la Agencia de Transformación Digital del Gobierno del Estado de Morelos (ATDEM). Busca reducir la brecha digital y que la ciudadanía pueda comunicarse sin costo, consultar la programación cultural, realizar trámites y acceder a las plataformas digitales institucionales.</t>
+          <t>El tamaño del círculo indica el número de computadoras. Haz clic en una escuela para ver su detalle.</t>
         </is>
       </c>
       <c r="E258" s="5" t="inlineStr">
         <is>
-          <t>Matlatl Wi-Fi tlen nochi ueli kitekiutiskej, amo iga tomin uan tlapojtok, tlen kichiua Agencia de Transformación Digital ipan Kaltlayekana ipan Morelos (ATDEM). Guinegui ma moyekchiua tlen amo kipiaj internet uan ma tlatlaga ueliskej monotsaskej amo iga tomin, kitaskej iljuimej, kichiuaskej trámites uan kalakiskej ipan plataformas digitales iga Kaltlayekana.</t>
+          <t>Kenin ueyi yaualtik kinextia keski tepostlapoualli kipia. Xikpacho se kaltlamachtiloyan iga tikitas nochi.</t>
         </is>
       </c>
       <c r="F258" s="4" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
@@ -8554,12 +8554,12 @@
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>Internet gratuito y abierto</t>
+          <t>Computadoras por aula</t>
         </is>
       </c>
       <c r="E259" s="5" t="inlineStr">
         <is>
-          <t>Internet amo iga tomin uan tlapojtok</t>
+          <t>Tepostlapoualli ipan nochi tlamachtiloyan</t>
         </is>
       </c>
       <c r="F259" s="4" t="inlineStr">
@@ -8575,7 +8575,7 @@
       </c>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C260" s="4" t="inlineStr">
@@ -8585,12 +8585,12 @@
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>Conexión Wi-Fi sin costo para la ciudadanía en espacios públicos y oficinas de gobierno.</t>
+          <t>Municipio con aula</t>
         </is>
       </c>
       <c r="E260" s="5" t="inlineStr">
         <is>
-          <t>Matlatl Wi-Fi amo iga tomin iga tlatlaga kanin nochi monechikouaj uan ipan teguichiualoyan iga Kaltlayekana.</t>
+          <t>Altepetl iga tlamachtiloyan</t>
         </is>
       </c>
       <c r="F260" s="4" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr">
@@ -8616,12 +8616,12 @@
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>Reducir la brecha digital</t>
+          <t>Otros municipios</t>
         </is>
       </c>
       <c r="E261" s="5" t="inlineStr">
         <is>
-          <t>Moyekchiuas tlen amo kipiaj internet</t>
+          <t>Siguin altepemej</t>
         </is>
       </c>
       <c r="F261" s="4" t="inlineStr">
@@ -8637,7 +8637,7 @@
       </c>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr">
@@ -8647,12 +8647,12 @@
       </c>
       <c r="D262" s="4" t="inlineStr">
         <is>
-          <t>Comunicarse sin costo, consultar programación cultural y realizar trámites en plataformas digitales institucionales.</t>
+          <t>Equipos por Municipio</t>
         </is>
       </c>
       <c r="E262" s="5" t="inlineStr">
         <is>
-          <t>Monotsaskej amo iga tomin, kitaskej iljuimej uan kichiuaskej trámites ipan plataformas digitales iga Kaltlayekana.</t>
+          <t>Tepostlapoualli iga altepetl</t>
         </is>
       </c>
       <c r="F262" s="4" t="inlineStr">
@@ -8668,7 +8668,7 @@
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
@@ -8678,12 +8678,12 @@
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>Puntos de conexión</t>
+          <t>{n} eq. · {n} esc.</t>
         </is>
       </c>
       <c r="E263" s="5" t="inlineStr">
         <is>
-          <t>Kanin mosaloua</t>
+          <t>{n} tep. · {n} kal.</t>
         </is>
       </c>
       <c r="F263" s="4" t="inlineStr">
@@ -8699,7 +8699,7 @@
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="D264" s="4" t="inlineStr">
         <is>
-          <t>Plazas públicas y espacios de alta concurrencia, como la Plaza de Armas Emiliano Zapata (Zócalo de Cuernavaca).</t>
+          <t>Escuelas</t>
         </is>
       </c>
       <c r="E264" s="5" t="inlineStr">
         <is>
-          <t>Plazas uan kanin miak tlatlaga monechikouaj, ken Plaza de Armas Emiliano Zapata (Zócalo de Cuernavaca).</t>
+          <t>Kaltlamachtiloyan</t>
         </is>
       </c>
       <c r="F264" s="4" t="inlineStr">
@@ -8730,7 +8730,7 @@
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
@@ -8740,12 +8740,12 @@
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>Eventos especiales, como el Festival Internacional Cervantino en Cuernavaca.</t>
+          <t>Escuela</t>
         </is>
       </c>
       <c r="E265" s="5" t="inlineStr">
         <is>
-          <t>Iljuimej, ken Festival Internacional Cervantino ipan Cuernavaca.</t>
+          <t>Kaltlamachtiloyan</t>
         </is>
       </c>
       <c r="F265" s="4" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr">
@@ -8771,12 +8771,12 @@
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>Dependencias estatales, ayudantías municipales y escuelas.</t>
+          <t>Equipos</t>
         </is>
       </c>
       <c r="E266" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga Kaltlayekana, ayudantías ipan altepemej uan kaltlamachtiloyan.</t>
+          <t>Tepostlapoualmej</t>
         </is>
       </c>
       <c r="F266" s="4" t="inlineStr">
@@ -8792,22 +8792,22 @@
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
         <is>
-          <t>Dependencias con red</t>
+          <t>Ver {d} en el mapa</t>
         </is>
       </c>
       <c r="E267" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga matlatl</t>
+          <t>Xikita {d} ipan tlalamatl</t>
         </is>
       </c>
       <c r="F267" s="4" t="inlineStr">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>Red La tierra que nos une</t>
+          <t>Aulas Tecnológicas</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr">
@@ -8833,12 +8833,12 @@
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>Secretarías y órganos</t>
+          <t>Fuente: ATDEM, "Proyecto Escuelas entrega Computadoras" (hoja Concentrado). Ubicación según el enlace de Google Maps capturado por escuela.</t>
         </is>
       </c>
       <c r="E268" s="5" t="inlineStr">
         <is>
-          <t>Secretarías uan teguichiualoyan</t>
+          <t>Kanin eua: ATDEM, "Proyecto Escuelas entrega Computadoras" (hoja Concentrado). Kanin katej iga ojtle Google Maps tlen motlalij iga nochi kaltlamachtiloyan.</t>
         </is>
       </c>
       <c r="F268" s="4" t="inlineStr">
@@ -8864,12 +8864,12 @@
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Sedes conectadas</t>
+          <t>Conectividad pública · Agencia de Transformación Digital</t>
         </is>
       </c>
       <c r="E269" s="5" t="inlineStr">
         <is>
-          <t>Kalmej tlen mosalojtokej</t>
+          <t>Matlatl tlapojtok · Agencia de Transformación Digital</t>
         </is>
       </c>
       <c r="F269" s="4" t="inlineStr">
@@ -8895,12 +8895,12 @@
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>Puntos de acceso</t>
+          <t>Red de Wi-Fi pública, gratuita y abierta impulsada por la Agencia de Transformación Digital del Gobierno del Estado de Morelos (ATDEM). Busca reducir la brecha digital y que la ciudadanía pueda comunicarse sin costo, consultar la programación cultural, realizar trámites y acceder a las plataformas digitales institucionales.</t>
         </is>
       </c>
       <c r="E270" s="5" t="inlineStr">
         <is>
-          <t>Kanin mosaloua</t>
+          <t>Matlatl Wi-Fi tlen nochi ueli kitekiutiskej, amo iga tomin uan tlapojtok, tlen kichiua Agencia de Transformación Digital ipan Kaltlayekana ipan Morelos (ATDEM). Guinegui ma moyekchiua tlen amo kipiaj internet uan ma tlatlaga ueliskej monotsaskej amo iga tomin, kitaskej iljuimej, kichiuaskej trámites uan kalakiskej ipan plataformas digitales iga Kaltlayekana.</t>
         </is>
       </c>
       <c r="F270" s="4" t="inlineStr">
@@ -8926,12 +8926,12 @@
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Mapa de la red</t>
+          <t>Internet gratuito y abierto</t>
         </is>
       </c>
       <c r="E271" s="5" t="inlineStr">
         <is>
-          <t>Tlalamatl iga matlatl</t>
+          <t>Internet amo iga tomin uan tlapojtok</t>
         </is>
       </c>
       <c r="F271" s="4" t="inlineStr">
@@ -8957,12 +8957,12 @@
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>Sede con red (el tamaño indica cuántas dependencias)</t>
+          <t>Conexión Wi-Fi sin costo para la ciudadanía en espacios públicos y oficinas de gobierno.</t>
         </is>
       </c>
       <c r="E272" s="5" t="inlineStr">
         <is>
-          <t>Kalle iga matlatl (kenin ueyi kinextia keski teguichiualoyan)</t>
+          <t>Matlatl Wi-Fi amo iga tomin iga tlatlaga kanin nochi monechikouaj uan ipan teguichiualoyan iga Kaltlayekana.</t>
         </is>
       </c>
       <c r="F272" s="4" t="inlineStr">
@@ -8988,12 +8988,12 @@
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>Dependencias por secretaría</t>
+          <t>Reducir la brecha digital</t>
         </is>
       </c>
       <c r="E273" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga secretaría</t>
+          <t>Moyekchiuas tlen amo kipiaj internet</t>
         </is>
       </c>
       <c r="F273" s="4" t="inlineStr">
@@ -9019,12 +9019,12 @@
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>{n} puntos de acceso</t>
+          <t>Comunicarse sin costo, consultar programación cultural y realizar trámites en plataformas digitales institucionales.</t>
         </is>
       </c>
       <c r="E274" s="5" t="inlineStr">
         <is>
-          <t>{n} kanin mosaloua</t>
+          <t>Monotsaskej amo iga tomin, kitaskej iljuimej uan kichiuaskej trámites ipan plataformas digitales iga Kaltlayekana.</t>
         </is>
       </c>
       <c r="F274" s="4" t="inlineStr">
@@ -9050,16 +9050,20 @@
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>Jefatura de la Oficina de la Gubernatura</t>
-        </is>
-      </c>
-      <c r="E275" s="4" t="n"/>
-      <c r="F275" s="4" t="n"/>
-      <c r="G275" s="4" t="inlineStr">
-        <is>
-          <t>Nombre propio o préstamo: se deja en español (confirmar).</t>
-        </is>
-      </c>
+          <t>Puntos de conexión</t>
+        </is>
+      </c>
+      <c r="E275" s="5" t="inlineStr">
+        <is>
+          <t>Kanin mosaloua</t>
+        </is>
+      </c>
+      <c r="F275" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n">
@@ -9077,12 +9081,12 @@
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>{n} punto de acceso</t>
+          <t>Plazas públicas y espacios de alta concurrencia, como la Plaza de Armas Emiliano Zapata (Zócalo de Cuernavaca).</t>
         </is>
       </c>
       <c r="E276" s="5" t="inlineStr">
         <is>
-          <t>{n} kanin mosaloua</t>
+          <t>Plazas uan kanin miak tlatlaga monechikouaj, ken Plaza de Armas Emiliano Zapata (Zócalo de Cuernavaca).</t>
         </is>
       </c>
       <c r="F276" s="4" t="inlineStr">
@@ -9108,12 +9112,12 @@
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (dependencias con red La tierra que nos une). Puntos de acceso según el registro de la ATDEM; algunas dependencias no tienen el dato capturado.</t>
+          <t>Eventos especiales, como el Festival Internacional Cervantino en Cuernavaca.</t>
         </is>
       </c>
       <c r="E277" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (teguichiualoyan iga matlatl Nin tlale tech sepaneloa). Kanin mosaloua ken kijkuiloj ATDEM; siguin teguichiualoyan amo kipiaj nin tlapoualli.</t>
+          <t>Iljuimej, ken Festival Internacional Cervantino ipan Cuernavaca.</t>
         </is>
       </c>
       <c r="F277" s="4" t="inlineStr">
@@ -9129,7 +9133,7 @@
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
@@ -9139,12 +9143,12 @@
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>Conectividad · Agencia de Transformación Digital</t>
+          <t>Dependencias estatales, ayudantías municipales y escuelas.</t>
         </is>
       </c>
       <c r="E278" s="5" t="inlineStr">
         <is>
-          <t>Mosaloua · Agencia de Transformación Digital</t>
+          <t>Teguichiualoyan iga Kaltlayekana, ayudantías ipan altepemej uan kaltlamachtiloyan.</t>
         </is>
       </c>
       <c r="F278" s="4" t="inlineStr">
@@ -9160,7 +9164,7 @@
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
@@ -9170,12 +9174,12 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>Sitios y torres de telecomunicaciones de la red estatal (sitios REEM) que dan servicio a dependencias del Gobierno del Estado, planteles educativos, unidades de salud e instalaciones de seguridad en Morelos.</t>
+          <t>Dependencias con red</t>
         </is>
       </c>
       <c r="E279" s="5" t="inlineStr">
         <is>
-          <t>Sitios uan tepostlaketsalmej iga uejka tlanonotsalistle ipan imatlau Kaltlayekana (sitios REEM) tlen kinpaleuiaj teguichiualoyan iga Kaltlayekana, kaltlamachtiloyan, pajtiloyan uan kanin tlajpiaj ipan Morelos.</t>
+          <t>Teguichiualoyan iga matlatl</t>
         </is>
       </c>
       <c r="F279" s="4" t="inlineStr">
@@ -9191,7 +9195,7 @@
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C280" s="4" t="inlineStr">
@@ -9201,12 +9205,12 @@
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>Por seguridad de la infraestructura, la información se presenta agregada por municipio y sector. No se publica la ubicación exacta ni el nombre de los sitios.</t>
+          <t>Secretarías y órganos</t>
         </is>
       </c>
       <c r="E280" s="5" t="inlineStr">
         <is>
-          <t>Iga tlajpialistle, tlamachilistle monextia sepan iga altepetl uan teguitl. Amo monextia kanin melauak katej nin intogayo sitios.</t>
+          <t>Secretarías uan teguichiualoyan</t>
         </is>
       </c>
       <c r="F280" s="4" t="inlineStr">
@@ -9222,7 +9226,7 @@
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
@@ -9232,12 +9236,12 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Sitios de telecomunicaciones</t>
+          <t>Sedes conectadas</t>
         </is>
       </c>
       <c r="E281" s="5" t="inlineStr">
         <is>
-          <t>Sitios iga uejka tlanonotsalistle</t>
+          <t>Kalmej tlen mosalojtokej</t>
         </is>
       </c>
       <c r="F281" s="4" t="inlineStr">
@@ -9253,7 +9257,7 @@
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr">
@@ -9263,12 +9267,12 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Municipios con sitios</t>
+          <t>Puntos de acceso</t>
         </is>
       </c>
       <c r="E282" s="5" t="inlineStr">
         <is>
-          <t>Altepemej iga sitios</t>
+          <t>Kanin mosaloua</t>
         </is>
       </c>
       <c r="F282" s="4" t="inlineStr">
@@ -9284,7 +9288,7 @@
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
@@ -9294,12 +9298,12 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Sectores atendidos</t>
+          <t>Mapa de la red</t>
         </is>
       </c>
       <c r="E283" s="5" t="inlineStr">
         <is>
-          <t>Teguimej tlen kinpaleuiaj</t>
+          <t>Tlalamatl iga matlatl</t>
         </is>
       </c>
       <c r="F283" s="4" t="inlineStr">
@@ -9315,7 +9319,7 @@
       </c>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr">
@@ -9325,12 +9329,12 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Mayor concentración ({n} sitios)</t>
+          <t>Sede con red (el tamaño indica cuántas dependencias)</t>
         </is>
       </c>
       <c r="E284" s="5" t="inlineStr">
         <is>
-          <t>Kanin ogachi miak ({n} sitios)</t>
+          <t>Kalle iga matlatl (kenin ueyi kinextia keski teguichiualoyan)</t>
         </is>
       </c>
       <c r="F284" s="4" t="inlineStr">
@@ -9346,7 +9350,7 @@
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
@@ -9356,12 +9360,12 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Sitios por municipio</t>
+          <t>Dependencias por secretaría</t>
         </is>
       </c>
       <c r="E285" s="5" t="inlineStr">
         <is>
-          <t>Sitios iga altepetl</t>
+          <t>Teguichiualoyan iga secretaría</t>
         </is>
       </c>
       <c r="F285" s="4" t="inlineStr">
@@ -9377,7 +9381,7 @@
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr">
@@ -9387,12 +9391,12 @@
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>Pasa el cursor sobre un municipio para ver el desglose por sector.</t>
+          <t>{n} puntos de acceso</t>
         </is>
       </c>
       <c r="E286" s="5" t="inlineStr">
         <is>
-          <t>Xikpano tepostlapacholi ipan se altepetl iga tikitas tlen kipia iga teguitl.</t>
+          <t>{n} kanin mosaloua</t>
         </is>
       </c>
       <c r="F286" s="4" t="inlineStr">
@@ -9408,7 +9412,7 @@
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
@@ -9418,20 +9422,16 @@
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>{n} o más</t>
-        </is>
-      </c>
-      <c r="E287" s="5" t="inlineStr">
-        <is>
-          <t>{n} o ogachi</t>
-        </is>
-      </c>
-      <c r="F287" s="4" t="inlineStr">
-        <is>
-          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
-        </is>
-      </c>
-      <c r="G287" s="4" t="n"/>
+          <t>Jefatura de la Oficina de la Gubernatura</t>
+        </is>
+      </c>
+      <c r="E287" s="4" t="n"/>
+      <c r="F287" s="4" t="n"/>
+      <c r="G287" s="4" t="inlineStr">
+        <is>
+          <t>Nombre propio o préstamo: se deja en español (confirmar).</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n">
@@ -9439,7 +9439,7 @@
       </c>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr">
@@ -9449,12 +9449,12 @@
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>Sin sitios</t>
+          <t>{n} punto de acceso</t>
         </is>
       </c>
       <c r="E288" s="5" t="inlineStr">
         <is>
-          <t>Amo kipia sitios</t>
+          <t>{n} kanin mosaloua</t>
         </is>
       </c>
       <c r="F288" s="4" t="inlineStr">
@@ -9470,7 +9470,7 @@
       </c>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr">
@@ -9480,12 +9480,12 @@
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Sitios por sector</t>
+          <t>Fuente: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (dependencias con red La tierra que nos une). Puntos de acceso según el registro de la ATDEM; algunas dependencias no tienen el dato capturado.</t>
         </is>
       </c>
       <c r="E289" s="5" t="inlineStr">
         <is>
-          <t>Sitios iga teguitl</t>
+          <t>Kanin eua: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (teguichiualoyan iga matlatl Nin tlale tech sepaneloa). Kanin mosaloua ken kijkuiloj ATDEM; siguin teguichiualoyan amo kipiaj nin tlapoualli.</t>
         </is>
       </c>
       <c r="F289" s="4" t="inlineStr">
@@ -9511,12 +9511,12 @@
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Gobierno del Estado</t>
+          <t>Conectividad · Agencia de Transformación Digital</t>
         </is>
       </c>
       <c r="E290" s="5" t="inlineStr">
         <is>
-          <t>Kaltlayekana</t>
+          <t>Mosaloua · Agencia de Transformación Digital</t>
         </is>
       </c>
       <c r="F290" s="4" t="inlineStr">
@@ -9542,12 +9542,12 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Sitios y torres de telecomunicaciones de la red estatal (sitios REEM) que dan servicio a dependencias del Gobierno del Estado, planteles educativos, unidades de salud e instalaciones de seguridad en Morelos.</t>
         </is>
       </c>
       <c r="E291" s="5" t="inlineStr">
         <is>
-          <t>Pajtilistle</t>
+          <t>Sitios uan tepostlaketsalmej iga uejka tlanonotsalistle ipan imatlau Kaltlayekana (sitios REEM) tlen kinpaleuiaj teguichiualoyan iga Kaltlayekana, kaltlamachtiloyan, pajtiloyan uan kanin tlajpiaj ipan Morelos.</t>
         </is>
       </c>
       <c r="F291" s="4" t="inlineStr">
@@ -9573,12 +9573,12 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Seguridad y Protección Ciudadana</t>
+          <t>Por seguridad de la infraestructura, la información se presenta agregada por municipio y sector. No se publica la ubicación exacta ni el nombre de los sitios.</t>
         </is>
       </c>
       <c r="E292" s="5" t="inlineStr">
         <is>
-          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga</t>
+          <t>Iga tlajpialistle, tlamachilistle monextia sepan iga altepetl uan teguitl. Amo monextia kanin melauak katej nin intogayo sitios.</t>
         </is>
       </c>
       <c r="F292" s="4" t="inlineStr">
@@ -9604,12 +9604,12 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Municipios con infraestructura</t>
+          <t>Sitios de telecomunicaciones</t>
         </is>
       </c>
       <c r="E293" s="5" t="inlineStr">
         <is>
-          <t>Altepemej iga tepostlaketsalmej</t>
+          <t>Sitios iga uejka tlanonotsalistle</t>
         </is>
       </c>
       <c r="F293" s="4" t="inlineStr">
@@ -9635,12 +9635,12 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Sectores</t>
+          <t>Municipios con sitios</t>
         </is>
       </c>
       <c r="E294" s="5" t="inlineStr">
         <is>
-          <t>Teguimej</t>
+          <t>Altepemej iga sitios</t>
         </is>
       </c>
       <c r="F294" s="4" t="inlineStr">
@@ -9666,12 +9666,12 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Sitios</t>
+          <t>Sectores atendidos</t>
         </is>
       </c>
       <c r="E295" s="5" t="inlineStr">
         <is>
-          <t>Sitios</t>
+          <t>Teguimej tlen kinpaleuiaj</t>
         </is>
       </c>
       <c r="F295" s="4" t="inlineStr">
@@ -9697,12 +9697,12 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Gobierno del Estado · {n}</t>
+          <t>Mayor concentración ({n} sitios)</t>
         </is>
       </c>
       <c r="E296" s="5" t="inlineStr">
         <is>
-          <t>Kaltlayekana · {n}</t>
+          <t>Kanin ogachi miak ({n} sitios)</t>
         </is>
       </c>
       <c r="F296" s="4" t="inlineStr">
@@ -9728,12 +9728,12 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>Salud · {n}</t>
+          <t>Sitios por municipio</t>
         </is>
       </c>
       <c r="E297" s="5" t="inlineStr">
         <is>
-          <t>Pajtilistle · {n}</t>
+          <t>Sitios iga altepetl</t>
         </is>
       </c>
       <c r="F297" s="4" t="inlineStr">
@@ -9759,12 +9759,12 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Educación · {n}</t>
+          <t>Pasa el cursor sobre un municipio para ver el desglose por sector.</t>
         </is>
       </c>
       <c r="E298" s="5" t="inlineStr">
         <is>
-          <t>Temachtilistle · {n}</t>
+          <t>Xikpano tepostlapacholi ipan se altepetl iga tikitas tlen kipia iga teguitl.</t>
         </is>
       </c>
       <c r="F298" s="4" t="inlineStr">
@@ -9790,12 +9790,12 @@
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>Seguridad y Protección Ciudadana · {n}</t>
+          <t>{n} o más</t>
         </is>
       </c>
       <c r="E299" s="5" t="inlineStr">
         <is>
-          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga · {n}</t>
+          <t>{n} o ogachi</t>
         </is>
       </c>
       <c r="F299" s="4" t="inlineStr">
@@ -9821,12 +9821,12 @@
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, registro de sitios REEM. Municipio asignado con los límites municipales del INE.</t>
+          <t>Sin sitios</t>
         </is>
       </c>
       <c r="E300" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, sitios REEM. Altepetl motlalij iga itlalxelol altepemej tlen INE.</t>
+          <t>Amo kipia sitios</t>
         </is>
       </c>
       <c r="F300" s="4" t="inlineStr">
@@ -9842,7 +9842,7 @@
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
@@ -9852,12 +9852,12 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Territorios de Paz y Buen Vivir · Transparencia</t>
+          <t>Sitios por sector</t>
         </is>
       </c>
       <c r="E301" s="5" t="inlineStr">
         <is>
-          <t>Territorios de Paz y Buen Vivir · Tlen nochi ueli kitaskej</t>
+          <t>Sitios iga teguitl</t>
         </is>
       </c>
       <c r="F301" s="4" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr">
@@ -9883,12 +9883,12 @@
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Descarga las bases de datos que alimentan este tablero. Cada conjunto está disponible en CSV, para abrirlo en Excel o cualquier herramienta de análisis, y en KML, para verlo en Google Earth o Google My Maps.</t>
+          <t>Gobierno del Estado</t>
         </is>
       </c>
       <c r="E302" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga tlapoualli tlen kitekiutia nin tablero. Nochi kipia CSV, iga tiktlapos ipan Excel o siguin programa, uan KML, iga tikitas ipan Google Earth o Google My Maps.</t>
+          <t>Kaltlayekana</t>
         </is>
       </c>
       <c r="F302" s="4" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr">
@@ -9914,12 +9914,12 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>{n} conjuntos de datos</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="E303" s="5" t="inlineStr">
         <is>
-          <t>{n} tlapoualamatl</t>
+          <t>Pajtilistle</t>
         </is>
       </c>
       <c r="F303" s="4" t="inlineStr">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
@@ -9945,12 +9945,12 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>CSV · UTF-{n}, separado por comas</t>
+          <t>Seguridad y Protección Ciudadana</t>
         </is>
       </c>
       <c r="E304" s="5" t="inlineStr">
         <is>
-          <t>CSV · UTF-{n}, xeloltok iga comas</t>
+          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga</t>
         </is>
       </c>
       <c r="F304" s="4" t="inlineStr">
@@ -9966,7 +9966,7 @@
       </c>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr">
@@ -9976,12 +9976,12 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>KML · una sola capa</t>
+          <t>Municipios con infraestructura</t>
         </is>
       </c>
       <c r="E305" s="5" t="inlineStr">
         <is>
-          <t>KML · san se tlapachtli</t>
+          <t>Altepemej iga tepostlaketsalmej</t>
         </is>
       </c>
       <c r="F305" s="4" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr">
@@ -10007,12 +10007,12 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Localidades · Propuesta Actual</t>
+          <t>Sectores</t>
         </is>
       </c>
       <c r="E306" s="5" t="inlineStr">
         <is>
-          <t>Altepetsitsin · Tlen axan</t>
+          <t>Teguimej</t>
         </is>
       </c>
       <c r="F306" s="4" t="inlineStr">
@@ -10028,7 +10028,7 @@
       </c>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr">
@@ -10038,12 +10038,12 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>{n} registros · {n} campos</t>
+          <t>Sitios</t>
         </is>
       </c>
       <c r="E307" s="5" t="inlineStr">
         <is>
-          <t>{n} tlajkuilolli · {n} tlamachilistle</t>
+          <t>Sitios</t>
         </is>
       </c>
       <c r="F307" s="4" t="inlineStr">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr">
@@ -10069,12 +10069,12 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Las localidades de los {n} polígonos vigentes con sus indicadores de población, vivienda, salud, educación, economía y marginación.</t>
+          <t>Gobierno del Estado · {n}</t>
         </is>
       </c>
       <c r="E308" s="5" t="inlineStr">
         <is>
-          <t>Altepetsitsin tlen {n} polígono tlen axan iga itlapoual tlatlaga, kalmej, pajtilistle, temachtilistle, tomin uan iknoyotl.</t>
+          <t>Kaltlayekana · {n}</t>
         </is>
       </c>
       <c r="F308" s="4" t="inlineStr">
@@ -10090,7 +10090,7 @@
       </c>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr">
@@ -10100,12 +10100,12 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Fuente: INEGI, Censo {n} (ITER Morelos) y Lista de Comunidades TPBV {n}</t>
+          <t>Salud · {n}</t>
         </is>
       </c>
       <c r="E309" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: INEGI, Censo {n} (ITER Morelos) uan Lista de Comunidades TPBV {n}</t>
+          <t>Pajtilistle · {n}</t>
         </is>
       </c>
       <c r="F309" s="4" t="inlineStr">
@@ -10121,7 +10121,7 @@
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr">
@@ -10131,12 +10131,12 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Ver campos</t>
+          <t>Educación · {n}</t>
         </is>
       </c>
       <c r="E310" s="5" t="inlineStr">
         <is>
-          <t>Xikita tlen kipia</t>
+          <t>Temachtilistle · {n}</t>
         </is>
       </c>
       <c r="F310" s="4" t="inlineStr">
@@ -10152,22 +10152,22 @@
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Descargar Localidades · Propuesta Actual en CSV</t>
+          <t>Seguridad y Protección Ciudadana · {n}</t>
         </is>
       </c>
       <c r="E311" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Altepetsitsin · Tlen axan ipan CSV</t>
+          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga · {n}</t>
         </is>
       </c>
       <c r="F311" s="4" t="inlineStr">
@@ -10183,22 +10183,22 @@
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Descargar Localidades · Propuesta Actual en KML</t>
+          <t>Fuente: ATDEM, registro de sitios REEM. Municipio asignado con los límites municipales del INE.</t>
         </is>
       </c>
       <c r="E312" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Altepetsitsin · Tlen axan ipan KML</t>
+          <t>Kanin eua: ATDEM, sitios REEM. Altepetl motlalij iga itlalxelol altepemej tlen INE.</t>
         </is>
       </c>
       <c r="F312" s="4" t="inlineStr">
@@ -10224,12 +10224,12 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Polígonos · Propuesta Actual</t>
+          <t>Territorios de Paz y Buen Vivir · Transparencia</t>
         </is>
       </c>
       <c r="E313" s="5" t="inlineStr">
         <is>
-          <t>Polígono · Tlen axan</t>
+          <t>Territorios de Paz y Buen Vivir · Tlen nochi ueli kitaskej</t>
         </is>
       </c>
       <c r="F313" s="4" t="inlineStr">
@@ -10255,12 +10255,12 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Contorno de los {n} polígonos vigentes de Territorios de Paz y Buen Vivir, con número de localidades y población.</t>
+          <t>Descarga las bases de datos que alimentan este tablero. Cada conjunto está disponible en CSV, para abrirlo en Excel o cualquier herramienta de análisis, y en KML, para verlo en Google Earth o Google My Maps.</t>
         </is>
       </c>
       <c r="E314" s="5" t="inlineStr">
         <is>
-          <t>Itlalxelol {n} polígono tlen axan ipan Territorios de Paz y Buen Vivir, iga keski altepetsitsin uan tlatlaga.</t>
+          <t>Xikuiga tlapoualli tlen kitekiutia nin tablero. Nochi kipia CSV, iga tiktlapos ipan Excel o siguin programa, uan KML, iga tikitas ipan Google Earth o Google My Maps.</t>
         </is>
       </c>
       <c r="F314" s="4" t="inlineStr">
@@ -10286,12 +10286,12 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Fuente: TPBV {n}.geojson</t>
+          <t>{n} conjuntos de datos</t>
         </is>
       </c>
       <c r="E315" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: TPBV {n}.geojson</t>
+          <t>{n} tlapoualamatl</t>
         </is>
       </c>
       <c r="F315" s="4" t="inlineStr">
@@ -10312,17 +10312,17 @@
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Descargar Polígonos · Propuesta Actual en CSV</t>
+          <t>CSV · UTF-{n}, separado por comas</t>
         </is>
       </c>
       <c r="E316" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Polígono · Tlen axan ipan CSV</t>
+          <t>CSV · UTF-{n}, xeloltok iga comas</t>
         </is>
       </c>
       <c r="F316" s="4" t="inlineStr">
@@ -10343,17 +10343,17 @@
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Descargar Polígonos · Propuesta Actual en KML</t>
+          <t>KML · una sola capa</t>
         </is>
       </c>
       <c r="E317" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Polígono · Tlen axan ipan KML</t>
+          <t>KML · san se tlapachtli</t>
         </is>
       </c>
       <c r="F317" s="4" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Escuelas donde ATDEM instaló aulas de cómputo: CCT, nivel, computadoras, fecha de instalación y polígono TPBV.</t>
+          <t>Localidades · Propuesta Actual</t>
         </is>
       </c>
       <c r="E318" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan kanin ATDEM kitlalij tepostlapoualli: CCT, temachtilistle, tepostlapoualmej, kemanian motlalij uan polígono TPBV.</t>
+          <t>Altepetsitsin · Tlen axan</t>
         </is>
       </c>
       <c r="F318" s="4" t="inlineStr">
@@ -10410,12 +10410,12 @@
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, Proyecto Escuelas entrega Computadoras</t>
+          <t>{n} registros · {n} campos</t>
         </is>
       </c>
       <c r="E319" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, Proyecto Escuelas entrega Computadoras</t>
+          <t>{n} tlajkuilolli · {n} tlamachilistle</t>
         </is>
       </c>
       <c r="F319" s="4" t="inlineStr">
@@ -10436,17 +10436,17 @@
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Descargar Aulas Tecnológicas en CSV</t>
+          <t>Las localidades de los {n} polígonos vigentes con sus indicadores de población, vivienda, salud, educación, economía y marginación.</t>
         </is>
       </c>
       <c r="E320" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan CSV</t>
+          <t>Altepetsitsin tlen {n} polígono tlen axan iga itlapoual tlatlaga, kalmej, pajtilistle, temachtilistle, tomin uan iknoyotl.</t>
         </is>
       </c>
       <c r="F320" s="4" t="inlineStr">
@@ -10467,17 +10467,17 @@
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Descargar Aulas Tecnológicas en KML</t>
+          <t>Fuente: INEGI, Censo {n} (ITER Morelos) y Lista de Comunidades TPBV {n}</t>
         </is>
       </c>
       <c r="E321" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan KML</t>
+          <t>Kanin eua: INEGI, Censo {n} (ITER Morelos) uan Lista de Comunidades TPBV {n}</t>
         </is>
       </c>
       <c r="F321" s="4" t="inlineStr">
@@ -10503,12 +10503,12 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Dependencias estatales con la red Wi-Fi pública de la ATDEM: secretaría, sede, coordenadas y puntos de acceso.</t>
+          <t>Ver campos</t>
         </is>
       </c>
       <c r="E322" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga Kaltlayekana tlen kipiaj matlatl Wi-Fi tlen ATDEM: secretaría, kalle, kanin katej uan kanin mosaloua.</t>
+          <t>Xikita tlen kipia</t>
         </is>
       </c>
       <c r="F322" s="4" t="inlineStr">
@@ -10529,17 +10529,17 @@
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+          <t>Descargar Localidades · Propuesta Actual en CSV</t>
         </is>
       </c>
       <c r="E323" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+          <t>Xikuiga Altepetsitsin · Tlen axan ipan CSV</t>
         </is>
       </c>
       <c r="F323" s="4" t="inlineStr">
@@ -10565,12 +10565,12 @@
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Descargar Red La tierra que nos une en CSV</t>
+          <t>Descargar Localidades · Propuesta Actual en KML</t>
         </is>
       </c>
       <c r="E324" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan CSV</t>
+          <t>Xikuiga Altepetsitsin · Tlen axan ipan KML</t>
         </is>
       </c>
       <c r="F324" s="4" t="inlineStr">
@@ -10591,17 +10591,17 @@
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Descargar Red La tierra que nos une en KML</t>
+          <t>Polígonos · Propuesta Actual</t>
         </is>
       </c>
       <c r="E325" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan KML</t>
+          <t>Polígono · Tlen axan</t>
         </is>
       </c>
       <c r="F325" s="4" t="inlineStr">
@@ -10627,12 +10627,12 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Límites municipales de Morelos</t>
+          <t>Contorno de los {n} polígonos vigentes de Territorios de Paz y Buen Vivir, con número de localidades y población.</t>
         </is>
       </c>
       <c r="E326" s="5" t="inlineStr">
         <is>
-          <t>Itlalxelol altepemej ipan Morelos</t>
+          <t>Itlalxelol {n} polígono tlen axan ipan Territorios de Paz y Buen Vivir, iga keski altepetsitsin uan tlatlaga.</t>
         </is>
       </c>
       <c r="F326" s="4" t="inlineStr">
@@ -10658,12 +10658,12 @@
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Contorno de los {n} municipios del estado, con clave geoestadística (CVEGEO) y nombre.</t>
+          <t>Fuente: TPBV {n}.geojson</t>
         </is>
       </c>
       <c r="E327" s="5" t="inlineStr">
         <is>
-          <t>Itlalxelol {n} altepemej, iga iclave geoestadística (CVEGEO) uan itoga.</t>
+          <t>Kanin eua: TPBV {n}.geojson</t>
         </is>
       </c>
       <c r="F327" s="4" t="inlineStr">
@@ -10684,17 +10684,17 @@
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Fuente: INE, límites municipales</t>
+          <t>Descargar Polígonos · Propuesta Actual en CSV</t>
         </is>
       </c>
       <c r="E328" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: INE, itlalxelol altepemej</t>
+          <t>Xikuiga Polígono · Tlen axan ipan CSV</t>
         </is>
       </c>
       <c r="F328" s="4" t="inlineStr">
@@ -10720,12 +10720,12 @@
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Descargar Límites municipales de Morelos en CSV</t>
+          <t>Descargar Polígonos · Propuesta Actual en KML</t>
         </is>
       </c>
       <c r="E329" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan CSV</t>
+          <t>Xikuiga Polígono · Tlen axan ipan KML</t>
         </is>
       </c>
       <c r="F329" s="4" t="inlineStr">
@@ -10746,17 +10746,17 @@
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Descargar Límites municipales de Morelos en KML</t>
+          <t>Escuelas donde ATDEM instaló aulas de cómputo: CCT, nivel, computadoras, fecha de instalación y polígono TPBV.</t>
         </is>
       </c>
       <c r="E330" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan KML</t>
+          <t>Kaltlamachtiloyan kanin ATDEM kitlalij tepostlapoualli: CCT, temachtilistle, tepostlapoualmej, kemanian motlalij uan polígono TPBV.</t>
         </is>
       </c>
       <c r="F330" s="4" t="inlineStr">
@@ -10782,12 +10782,12 @@
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Los archivos se generan en tu navegador con la misma información que muestra el tablero. Para Google My Maps importa el KML en una capa nueva y usa "Aplicar estilo por columna de datos" para colorear por municipio, polígono u otro campo.</t>
+          <t>Fuente: ATDEM, Proyecto Escuelas entrega Computadoras</t>
         </is>
       </c>
       <c r="E331" s="5" t="inlineStr">
         <is>
-          <t>Nin amatl mochiua ipan motepostlapoual iga nochi tlamachilistle tlen kinextia nin tablero. Iga Google My Maps, xikalaki KML ipan se yankuik tlapachtli uan xiktekiuti "Aplicar estilo por columna de datos" iga tiktlapaluis iga altepetl, polígono o siguin.</t>
+          <t>Kanin eua: ATDEM, Proyecto Escuelas entrega Computadoras</t>
         </is>
       </c>
       <c r="F331" s="4" t="inlineStr">
@@ -10803,22 +10803,22 @@
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>Inicio (buscador de comunidades)</t>
+          <t>Datos Abiertos</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>No encontramos «{d}» entre las {n} comunidades del programa. Revisa cómo está escrito o busca por municipio.</t>
+          <t>Descargar Aulas Tecnológicas en CSV</t>
         </is>
       </c>
       <c r="E332" s="5" t="inlineStr">
         <is>
-          <t>Amo otikajsike «{d}» ipan {n} altepetsitsin tlen nin tlapaleuilistle. Xiktlachili kenin otiktlajkuilo o xiktemo iga altepetl.</t>
+          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan CSV</t>
         </is>
       </c>
       <c r="F332" s="4" t="inlineStr">
@@ -10834,22 +10834,22 @@
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>Inicio (buscador de comunidades)</t>
+          <t>Datos Abiertos</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>{d} tiene {n} comunidad en el programa.</t>
+          <t>Descargar Aulas Tecnológicas en KML</t>
         </is>
       </c>
       <c r="E333" s="5" t="inlineStr">
         <is>
-          <t>{d} kipia {n} altepetsin ipan nin tlapaleuilistle.</t>
+          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan KML</t>
         </is>
       </c>
       <c r="F333" s="4" t="inlineStr">
@@ -10865,7 +10865,7 @@
       </c>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>Inicio (buscador de comunidades)</t>
+          <t>Datos Abiertos</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr">
@@ -10875,12 +10875,12 @@
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Y {n} comunidad más. Escribe más letras para afinar la búsqueda.</t>
+          <t>Dependencias estatales con la red Wi-Fi pública de la ATDEM: secretaría, sede, coordenadas y puntos de acceso.</t>
         </is>
       </c>
       <c r="E334" s="5" t="inlineStr">
         <is>
-          <t>Uan ogachi {n} altepetsin. Xiktlajkuilo ogachi tlajkuilolli iga tiktemos kuale.</t>
+          <t>Teguichiualoyan iga Kaltlayekana tlen kipiaj matlatl Wi-Fi tlen ATDEM: secretaría, kalle, kanin katej uan kanin mosaloua.</t>
         </is>
       </c>
       <c r="F334" s="4" t="inlineStr">
@@ -10896,33 +10896,405 @@
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C335" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D335" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+        </is>
+      </c>
+      <c r="E335" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+        </is>
+      </c>
+      <c r="F335" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G335" s="4" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="4" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C336" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D336" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Red La tierra que nos une en CSV</t>
+        </is>
+      </c>
+      <c r="E336" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan CSV</t>
+        </is>
+      </c>
+      <c r="F336" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G336" s="4" t="n"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="4" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C337" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D337" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Red La tierra que nos une en KML</t>
+        </is>
+      </c>
+      <c r="E337" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan KML</t>
+        </is>
+      </c>
+      <c r="F337" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G337" s="4" t="n"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="4" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C338" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D338" s="4" t="inlineStr">
+        <is>
+          <t>Límites municipales de Morelos</t>
+        </is>
+      </c>
+      <c r="E338" s="5" t="inlineStr">
+        <is>
+          <t>Itlalxelol altepemej ipan Morelos</t>
+        </is>
+      </c>
+      <c r="F338" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G338" s="4" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="4" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C339" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr">
+        <is>
+          <t>Contorno de los {n} municipios del estado, con clave geoestadística (CVEGEO) y nombre.</t>
+        </is>
+      </c>
+      <c r="E339" s="5" t="inlineStr">
+        <is>
+          <t>Itlalxelol {n} altepemej, iga iclave geoestadística (CVEGEO) uan itoga.</t>
+        </is>
+      </c>
+      <c r="F339" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G339" s="4" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="4" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C340" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D340" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: INE, límites municipales</t>
+        </is>
+      </c>
+      <c r="E340" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: INE, itlalxelol altepemej</t>
+        </is>
+      </c>
+      <c r="F340" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G340" s="4" t="n"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="4" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C341" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D341" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Límites municipales de Morelos en CSV</t>
+        </is>
+      </c>
+      <c r="E341" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan CSV</t>
+        </is>
+      </c>
+      <c r="F341" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G341" s="4" t="n"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="4" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D342" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Límites municipales de Morelos en KML</t>
+        </is>
+      </c>
+      <c r="E342" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan KML</t>
+        </is>
+      </c>
+      <c r="F342" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G342" s="4" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="4" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C343" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D343" s="4" t="inlineStr">
+        <is>
+          <t>Los archivos se generan en tu navegador con la misma información que muestra el tablero. Para Google My Maps importa el KML en una capa nueva y usa "Aplicar estilo por columna de datos" para colorear por municipio, polígono u otro campo.</t>
+        </is>
+      </c>
+      <c r="E343" s="5" t="inlineStr">
+        <is>
+          <t>Nin amatl mochiua ipan motepostlapoual iga nochi tlamachilistle tlen kinextia nin tablero. Iga Google My Maps, xikalaki KML ipan se yankuik tlapachtli uan xiktekiuti "Aplicar estilo por columna de datos" iga tiktlapaluis iga altepetl, polígono o siguin.</t>
+        </is>
+      </c>
+      <c r="F343" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G343" s="4" t="n"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="4" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" s="4" t="inlineStr">
+        <is>
+          <t>Inicio (buscador de comunidades)</t>
+        </is>
+      </c>
+      <c r="C344" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D344" s="4" t="inlineStr">
+        <is>
+          <t>No encontramos «{d}» entre las {n} comunidades del programa. Revisa cómo está escrito o busca por municipio.</t>
+        </is>
+      </c>
+      <c r="E344" s="5" t="inlineStr">
+        <is>
+          <t>Amo otikajsike «{d}» ipan {n} altepetsitsin tlen nin tlapaleuilistle. Xiktlachili kenin otiktlajkuilo o xiktemo iga altepetl.</t>
+        </is>
+      </c>
+      <c r="F344" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G344" s="4" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="4" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" s="4" t="inlineStr">
+        <is>
+          <t>Inicio (buscador de comunidades)</t>
+        </is>
+      </c>
+      <c r="C345" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D345" s="4" t="inlineStr">
+        <is>
+          <t>{d} tiene {n} comunidad en el programa.</t>
+        </is>
+      </c>
+      <c r="E345" s="5" t="inlineStr">
+        <is>
+          <t>{d} kipia {n} altepetsin ipan nin tlapaleuilistle.</t>
+        </is>
+      </c>
+      <c r="F345" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G345" s="4" t="n"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="4" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" s="4" t="inlineStr">
+        <is>
+          <t>Inicio (buscador de comunidades)</t>
+        </is>
+      </c>
+      <c r="C346" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D346" s="4" t="inlineStr">
+        <is>
+          <t>Y {n} comunidad más. Escribe más letras para afinar la búsqueda.</t>
+        </is>
+      </c>
+      <c r="E346" s="5" t="inlineStr">
+        <is>
+          <t>Uan ogachi {n} altepetsin. Xiktlajkuilo ogachi tlajkuilolli iga tiktemos kuale.</t>
+        </is>
+      </c>
+      <c r="F346" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G346" s="4" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="4" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" s="4" t="inlineStr">
+        <is>
           <t>Encabezado y menú</t>
         </is>
       </c>
-      <c r="C335" s="4" t="inlineStr">
+      <c r="C347" s="4" t="inlineStr">
         <is>
           <t>atributo</t>
         </is>
       </c>
-      <c r="D335" s="4" t="inlineStr">
+      <c r="D347" s="4" t="inlineStr">
         <is>
           <t>Territorios de Paz y Buen Vivir · Gobierno de Morelos</t>
         </is>
       </c>
-      <c r="E335" s="5" t="inlineStr">
+      <c r="E347" s="5" t="inlineStr">
         <is>
           <t>Territorios de Paz y Buen Vivir · Kaltlayekana ipan Morelos</t>
         </is>
       </c>
-      <c r="F335" s="4" t="inlineStr">
-        <is>
-          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
-        </is>
-      </c>
-      <c r="G335" s="4" t="n"/>
+      <c r="F347" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G347" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G335"/>
+  <autoFilter ref="A1:G347"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: WiFi en comunidades y carrusel en Red; oculta Telecomunicaciones
- Red La tierra que nos une: 11 comunidades (instalado / en proceso) en el
  mapa, cifras y lista; titulo "Disponibilidad de WiFi gratuito en oficinas
  de gobierno"; seccion de la nota del 07/08/2026 con carrusel de 4 fotos.
- Conjunto nuevo en Datos Abiertos (comunidades con red).
- Telecomunicaciones oculta por el momento (MOSTRAR_TELECOM = false).
- Sin numeros de ticket ni fechas del registro interno.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traducciones/Traduccion_nahuatl_tablero.xlsx
+++ b/traducciones/Traduccion_nahuatl_tablero.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$G$347</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Textos'!$A$1:$G$378</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G347"/>
+  <dimension ref="A1:G378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3963,12 +3963,12 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Mapa de las dependencias estatales que ya cuentan con la red Wi-Fi pública y gratuita de la ATDEM: sedes, secretarías y puntos de acceso.</t>
+          <t>Mapa de la red Wi-Fi pública y gratuita de la ATDEM en oficinas de gobierno y en comunidades: sedes, puntos de acceso y avance de instalación.</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>Tlalamatl iga teguichiualoyan iga Kaltlayekana tlen ya kipiaj matlatl Wi-Fi tlapojtok uan amo iga tomin tlen ATDEM: kalmej, secretarías uan kanin mosaloua.</t>
+          <t>Tlalamatl iga matlatl Wi-Fi tlapojtok uan amo iga tomin tlen ATDEM ipan teguichiualoyan iga Kaltlayekana uan ipan altepetsitsin: kalmej, kanin mosaloua uan kenin motlalijtiga.</t>
         </is>
       </c>
       <c r="F110" s="4" t="inlineStr">
@@ -9174,12 +9174,12 @@
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>Dependencias con red</t>
+          <t>{n} de agosto de {n} · Comunidades prioritarias</t>
         </is>
       </c>
       <c r="E279" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga matlatl</t>
+          <t>{n} agosto, {n} xiuitl · Altepetsitsin tlen achtopa</t>
         </is>
       </c>
       <c r="F279" s="4" t="inlineStr">
@@ -9205,12 +9205,12 @@
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>Secretarías y órganos</t>
+          <t>Internet gratuito en comunidades prioritarias</t>
         </is>
       </c>
       <c r="E280" s="5" t="inlineStr">
         <is>
-          <t>Secretarías uan teguichiualoyan</t>
+          <t>Internet amo iga tomin ipan altepetsitsin tlen achtopa</t>
         </is>
       </c>
       <c r="F280" s="4" t="inlineStr">
@@ -9236,12 +9236,12 @@
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>Sedes conectadas</t>
+          <t>La ATDEM amplía la red «La tierra que nos une» a zonas históricamente vulnerables. El servicio opera al cien por ciento en El Zapote ({d}) y en Villa Nicolás Zapata ({d}), con puntos Wi-Fi en plazas principales, centros comunitarios y planteles educativos, y personal técnico realiza estudios de factibilidad en {d} y otras localidades de Territorios de Paz y Buen Vivir.</t>
         </is>
       </c>
       <c r="E281" s="5" t="inlineStr">
         <is>
-          <t>Kalmej tlen mosalojtokej</t>
+          <t>ATDEM kiueyichiua matlatl «Nin tlale tech sepaneloa» ipan altepetsitsin tlen miak xiuitl amo kipiayaj. Matlatl ya nochi teguiti ipan El Zapote ({d}) uan ipan Villa Nicolás Zapata ({d}), iga Wi-Fi ipan plazas, kalmej tlen altepetsin uan kaltlamachtiloyan, uan tlatlaga tlen kimatij kitemoaj kenin uelis motlalis ipan {d} uan siguin altepetsitsin tlen Territorios de Paz y Buen Vivir.</t>
         </is>
       </c>
       <c r="F281" s="4" t="inlineStr">
@@ -9267,12 +9267,12 @@
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Puntos de acceso</t>
+          <t>comunidades con red instalada</t>
         </is>
       </c>
       <c r="E282" s="5" t="inlineStr">
         <is>
-          <t>Kanin mosaloua</t>
+          <t>altepetsitsin tlen ya kipiaj matlatl</t>
         </is>
       </c>
       <c r="F282" s="4" t="inlineStr">
@@ -9298,12 +9298,12 @@
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Mapa de la red</t>
+          <t>comunidades en proceso de instalación</t>
         </is>
       </c>
       <c r="E283" s="5" t="inlineStr">
         <is>
-          <t>Tlalamatl iga matlatl</t>
+          <t>altepetsitsin kanin matlatl motlalijtiga</t>
         </is>
       </c>
       <c r="F283" s="4" t="inlineStr">
@@ -9329,12 +9329,12 @@
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>Sede con red (el tamaño indica cuántas dependencias)</t>
+          <t>“El internet no puede seguir siendo un privilegio de pocos; es una herramienta de equidad social.”</t>
         </is>
       </c>
       <c r="E284" s="5" t="inlineStr">
         <is>
-          <t>Kalle iga matlatl (kenin ueyi kinextia keski teguichiualoyan)</t>
+          <t>“Internet amo ueli san sansiguin kipiaske; ika internet nochi sepan tiuejueyij.”</t>
         </is>
       </c>
       <c r="F284" s="4" t="inlineStr">
@@ -9360,12 +9360,12 @@
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>Dependencias por secretaría</t>
+          <t>Samuel Rivera Muciño, titular de la ATDEM</t>
         </is>
       </c>
       <c r="E285" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga secretaría</t>
+          <t>Samuel Rivera Muciño, tlayekanki ipan ATDEM</t>
         </is>
       </c>
       <c r="F285" s="4" t="inlineStr">
@@ -9386,17 +9386,17 @@
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>{n} puntos de acceso</t>
+          <t>Fotos de la red en comunidades prioritarias</t>
         </is>
       </c>
       <c r="E286" s="5" t="inlineStr">
         <is>
-          <t>{n} kanin mosaloua</t>
+          <t>Ixkopinkayomej tlen matlatl ipan altepetsitsin tlen achtopa</t>
         </is>
       </c>
       <c r="F286" s="4" t="inlineStr">
@@ -9417,21 +9417,25 @@
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>Jefatura de la Oficina de la Gubernatura</t>
-        </is>
-      </c>
-      <c r="E287" s="4" t="n"/>
-      <c r="F287" s="4" t="n"/>
-      <c r="G287" s="4" t="inlineStr">
-        <is>
-          <t>Nombre propio o préstamo: se deja en español (confirmar).</t>
-        </is>
-      </c>
+          <t>Personal técnico de la ATDEM durante un recorrido de campo.</t>
+        </is>
+      </c>
+      <c r="E287" s="5" t="inlineStr">
+        <is>
+          <t>Tlatlaga tlen ATDEM kuak nejnemij ipan tlale.</t>
+        </is>
+      </c>
+      <c r="F287" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n">
@@ -9444,17 +9448,17 @@
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>{n} punto de acceso</t>
+          <t>Visita de la ATDEM a un centro comunitario.</t>
         </is>
       </c>
       <c r="E288" s="5" t="inlineStr">
         <is>
-          <t>{n} kanin mosaloua</t>
+          <t>ATDEM kipaxaloua se kalle tlen altepetsin.</t>
         </is>
       </c>
       <c r="F288" s="4" t="inlineStr">
@@ -9475,17 +9479,17 @@
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (dependencias con red La tierra que nos une). Puntos de acceso según el registro de la ATDEM; algunas dependencias no tienen el dato capturado.</t>
+          <t>Infraestructura de telecomunicaciones para llevar la red a las comunidades.</t>
         </is>
       </c>
       <c r="E289" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (teguichiualoyan iga matlatl Nin tlale tech sepaneloa). Kanin mosaloua ken kijkuiloj ATDEM; siguin teguichiualoyan amo kipiaj nin tlapoualli.</t>
+          <t>Tepostlaketsalli iga kuiguiliske matlatl altepetsitsin.</t>
         </is>
       </c>
       <c r="F289" s="4" t="inlineStr">
@@ -9501,22 +9505,22 @@
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>atributo</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>Conectividad · Agencia de Transformación Digital</t>
+          <t>Estudios de factibilidad tecnológica en zonas prioritarias del estado.</t>
         </is>
       </c>
       <c r="E290" s="5" t="inlineStr">
         <is>
-          <t>Mosaloua · Agencia de Transformación Digital</t>
+          <t>Kitemoaj kenin uelis motlalis matlatl ipan altepetsitsin tlen achtopa.</t>
         </is>
       </c>
       <c r="F290" s="4" t="inlineStr">
@@ -9532,7 +9536,7 @@
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
@@ -9542,12 +9546,12 @@
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Sitios y torres de telecomunicaciones de la red estatal (sitios REEM) que dan servicio a dependencias del Gobierno del Estado, planteles educativos, unidades de salud e instalaciones de seguridad en Morelos.</t>
+          <t>Dependencias con red</t>
         </is>
       </c>
       <c r="E291" s="5" t="inlineStr">
         <is>
-          <t>Sitios uan tepostlaketsalmej iga uejka tlanonotsalistle ipan imatlau Kaltlayekana (sitios REEM) tlen kinpaleuiaj teguichiualoyan iga Kaltlayekana, kaltlamachtiloyan, pajtiloyan uan kanin tlajpiaj ipan Morelos.</t>
+          <t>Teguichiualoyan iga matlatl</t>
         </is>
       </c>
       <c r="F291" s="4" t="inlineStr">
@@ -9563,7 +9567,7 @@
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr">
@@ -9573,12 +9577,12 @@
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Por seguridad de la infraestructura, la información se presenta agregada por municipio y sector. No se publica la ubicación exacta ni el nombre de los sitios.</t>
+          <t>Secretarías y órganos</t>
         </is>
       </c>
       <c r="E292" s="5" t="inlineStr">
         <is>
-          <t>Iga tlajpialistle, tlamachilistle monextia sepan iga altepetl uan teguitl. Amo monextia kanin melauak katej nin intogayo sitios.</t>
+          <t>Secretarías uan teguichiualoyan</t>
         </is>
       </c>
       <c r="F292" s="4" t="inlineStr">
@@ -9594,7 +9598,7 @@
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
@@ -9604,12 +9608,12 @@
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Sitios de telecomunicaciones</t>
+          <t>Sedes conectadas</t>
         </is>
       </c>
       <c r="E293" s="5" t="inlineStr">
         <is>
-          <t>Sitios iga uejka tlanonotsalistle</t>
+          <t>Kalmej tlen mosalojtokej</t>
         </is>
       </c>
       <c r="F293" s="4" t="inlineStr">
@@ -9625,7 +9629,7 @@
       </c>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr">
@@ -9635,12 +9639,12 @@
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Municipios con sitios</t>
+          <t>Puntos de acceso</t>
         </is>
       </c>
       <c r="E294" s="5" t="inlineStr">
         <is>
-          <t>Altepemej iga sitios</t>
+          <t>Kanin mosaloua</t>
         </is>
       </c>
       <c r="F294" s="4" t="inlineStr">
@@ -9656,7 +9660,7 @@
       </c>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr">
@@ -9666,12 +9670,12 @@
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Sectores atendidos</t>
+          <t>WiFi gratuito en comunidades</t>
         </is>
       </c>
       <c r="E295" s="5" t="inlineStr">
         <is>
-          <t>Teguimej tlen kinpaleuiaj</t>
+          <t>WiFi amo iga tomin ipan altepetsitsin</t>
         </is>
       </c>
       <c r="F295" s="4" t="inlineStr">
@@ -9687,7 +9691,7 @@
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr">
@@ -9697,12 +9701,12 @@
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>Mayor concentración ({n} sitios)</t>
+          <t>Comunidades</t>
         </is>
       </c>
       <c r="E296" s="5" t="inlineStr">
         <is>
-          <t>Kanin ogachi miak ({n} sitios)</t>
+          <t>Altepetsitsin</t>
         </is>
       </c>
       <c r="F296" s="4" t="inlineStr">
@@ -9718,7 +9722,7 @@
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
@@ -9728,12 +9732,12 @@
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>Sitios por municipio</t>
+          <t>Con red instalada</t>
         </is>
       </c>
       <c r="E297" s="5" t="inlineStr">
         <is>
-          <t>Sitios iga altepetl</t>
+          <t>Ya kipiaj matlatl</t>
         </is>
       </c>
       <c r="F297" s="4" t="inlineStr">
@@ -9749,7 +9753,7 @@
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
@@ -9759,12 +9763,12 @@
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>Pasa el cursor sobre un municipio para ver el desglose por sector.</t>
+          <t>En proceso de instalación</t>
         </is>
       </c>
       <c r="E298" s="5" t="inlineStr">
         <is>
-          <t>Xikpano tepostlapacholi ipan se altepetl iga tikitas tlen kipia iga teguitl.</t>
+          <t>Matlatl motlalijtiga</t>
         </is>
       </c>
       <c r="F298" s="4" t="inlineStr">
@@ -9780,7 +9784,7 @@
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
@@ -9790,12 +9794,12 @@
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>{n} o más</t>
+          <t>En comunidades TPBV</t>
         </is>
       </c>
       <c r="E299" s="5" t="inlineStr">
         <is>
-          <t>{n} o ogachi</t>
+          <t>Ipan altepetsitsin TPBV</t>
         </is>
       </c>
       <c r="F299" s="4" t="inlineStr">
@@ -9811,7 +9815,7 @@
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
@@ -9821,12 +9825,12 @@
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>Sin sitios</t>
+          <t>Mapa de la red</t>
         </is>
       </c>
       <c r="E300" s="5" t="inlineStr">
         <is>
-          <t>Amo kipia sitios</t>
+          <t>Tlalamatl iga matlatl</t>
         </is>
       </c>
       <c r="F300" s="4" t="inlineStr">
@@ -9842,7 +9846,7 @@
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
@@ -9852,12 +9856,12 @@
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Sitios por sector</t>
+          <t>Oficina de gobierno (el tamaño indica cuántas dependencias)</t>
         </is>
       </c>
       <c r="E301" s="5" t="inlineStr">
         <is>
-          <t>Sitios iga teguitl</t>
+          <t>Teguichiualoyan iga Kaltlayekana (kenin ueyi kinextia keski teguichiualoyan)</t>
         </is>
       </c>
       <c r="F301" s="4" t="inlineStr">
@@ -9873,7 +9877,7 @@
       </c>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr">
@@ -9883,12 +9887,12 @@
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>Gobierno del Estado</t>
+          <t>Comunidad: instalado</t>
         </is>
       </c>
       <c r="E302" s="5" t="inlineStr">
         <is>
-          <t>Kaltlayekana</t>
+          <t>Altepetsin: motlalij</t>
         </is>
       </c>
       <c r="F302" s="4" t="inlineStr">
@@ -9904,7 +9908,7 @@
       </c>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr">
@@ -9914,12 +9918,12 @@
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Comunidad: en proceso</t>
         </is>
       </c>
       <c r="E303" s="5" t="inlineStr">
         <is>
-          <t>Pajtilistle</t>
+          <t>Altepetsin: motlalijtiga</t>
         </is>
       </c>
       <c r="F303" s="4" t="inlineStr">
@@ -9935,7 +9939,7 @@
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
@@ -9945,12 +9949,12 @@
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Seguridad y Protección Ciudadana</t>
+          <t>Instalado</t>
         </is>
       </c>
       <c r="E304" s="5" t="inlineStr">
         <is>
-          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga</t>
+          <t>Motlalij</t>
         </is>
       </c>
       <c r="F304" s="4" t="inlineStr">
@@ -9966,7 +9970,7 @@
       </c>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr">
@@ -9976,12 +9980,12 @@
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Municipios con infraestructura</t>
+          <t>{d} · Comunidad TPBV</t>
         </is>
       </c>
       <c r="E305" s="5" t="inlineStr">
         <is>
-          <t>Altepemej iga tepostlaketsalmej</t>
+          <t>{d} · Altepetsin TPBV</t>
         </is>
       </c>
       <c r="F305" s="4" t="inlineStr">
@@ -9997,7 +10001,7 @@
       </c>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr">
@@ -10007,12 +10011,12 @@
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Sectores</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="E306" s="5" t="inlineStr">
         <is>
-          <t>Teguimej</t>
+          <t>Motlalijtiga</t>
         </is>
       </c>
       <c r="F306" s="4" t="inlineStr">
@@ -10028,7 +10032,7 @@
       </c>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr">
@@ -10038,12 +10042,12 @@
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>Sitios</t>
+          <t>Disponibilidad de WiFi gratuito en oficinas de gobierno</t>
         </is>
       </c>
       <c r="E307" s="5" t="inlineStr">
         <is>
-          <t>Sitios</t>
+          <t>Kanin onka WiFi amo iga tomin ipan teguichiualoyan iga Kaltlayekana</t>
         </is>
       </c>
       <c r="F307" s="4" t="inlineStr">
@@ -10059,7 +10063,7 @@
       </c>
       <c r="B308" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C308" s="4" t="inlineStr">
@@ -10069,12 +10073,12 @@
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>Gobierno del Estado · {n}</t>
+          <t>{n} puntos de acceso</t>
         </is>
       </c>
       <c r="E308" s="5" t="inlineStr">
         <is>
-          <t>Kaltlayekana · {n}</t>
+          <t>{n} kanin mosaloua</t>
         </is>
       </c>
       <c r="F308" s="4" t="inlineStr">
@@ -10090,7 +10094,7 @@
       </c>
       <c r="B309" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C309" s="4" t="inlineStr">
@@ -10100,20 +10104,16 @@
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>Salud · {n}</t>
-        </is>
-      </c>
-      <c r="E309" s="5" t="inlineStr">
-        <is>
-          <t>Pajtilistle · {n}</t>
-        </is>
-      </c>
-      <c r="F309" s="4" t="inlineStr">
-        <is>
-          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
-        </is>
-      </c>
-      <c r="G309" s="4" t="n"/>
+          <t>Jefatura de la Oficina de la Gubernatura</t>
+        </is>
+      </c>
+      <c r="E309" s="4" t="n"/>
+      <c r="F309" s="4" t="n"/>
+      <c r="G309" s="4" t="inlineStr">
+        <is>
+          <t>Nombre propio o préstamo: se deja en español (confirmar).</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n">
@@ -10121,7 +10121,7 @@
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr">
@@ -10131,12 +10131,12 @@
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Educación · {n}</t>
+          <t>{n} punto de acceso</t>
         </is>
       </c>
       <c r="E310" s="5" t="inlineStr">
         <is>
-          <t>Temachtilistle · {n}</t>
+          <t>{n} kanin mosaloua</t>
         </is>
       </c>
       <c r="F310" s="4" t="inlineStr">
@@ -10152,7 +10152,7 @@
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
@@ -10162,12 +10162,12 @@
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Seguridad y Protección Ciudadana · {n}</t>
+          <t>Fuente: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (dependencias con red La tierra que nos une) y registro de instalaciones en comunidades. Puntos de acceso según el registro de la ATDEM; algunas dependencias no tienen el dato capturado.</t>
         </is>
       </c>
       <c r="E311" s="5" t="inlineStr">
         <is>
-          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga · {n}</t>
+          <t>Kanin eua: ATDEM, "Agentes_dependencias La Tierra Que Nos Une" (teguichiualoyan iga matlatl Nin tlale tech sepaneloa) uan itlajkuilol tlen motlalij ipan altepetsitsin. Kanin mosaloua ken kijkuiloj ATDEM; siguin teguichiualoyan amo kipiaj nin tlapoualli.</t>
         </is>
       </c>
       <c r="F311" s="4" t="inlineStr">
@@ -10183,7 +10183,7 @@
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura de Telecomunicaciones</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
@@ -10193,12 +10193,12 @@
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, registro de sitios REEM. Municipio asignado con los límites municipales del INE.</t>
+          <t>WiFi gratuito: instalado</t>
         </is>
       </c>
       <c r="E312" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, sitios REEM. Altepetl motlalij iga itlalxelol altepemej tlen INE.</t>
+          <t>WiFi amo iga tomin: motlalij</t>
         </is>
       </c>
       <c r="F312" s="4" t="inlineStr">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
@@ -10224,12 +10224,12 @@
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Territorios de Paz y Buen Vivir · Transparencia</t>
+          <t>Comunidad de Territorios de Paz y Buen Vivir · Polígono {d}</t>
         </is>
       </c>
       <c r="E313" s="5" t="inlineStr">
         <is>
-          <t>Territorios de Paz y Buen Vivir · Tlen nochi ueli kitaskej</t>
+          <t>Altepetsin ipan Territorios de Paz y Buen Vivir · Polígono {d}</t>
         </is>
       </c>
       <c r="F313" s="4" t="inlineStr">
@@ -10245,7 +10245,7 @@
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr">
@@ -10255,12 +10255,12 @@
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Descarga las bases de datos que alimentan este tablero. Cada conjunto está disponible en CSV, para abrirlo en Excel o cualquier herramienta de análisis, y en KML, para verlo en Google Earth o Google My Maps.</t>
+          <t>Ubicación aproximada de la localidad</t>
         </is>
       </c>
       <c r="E314" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga tlapoualli tlen kitekiutia nin tablero. Nochi kipia CSV, iga tiktlapos ipan Excel o siguin programa, uan KML, iga tikitas ipan Google Earth o Google My Maps.</t>
+          <t>Kanin katej altepetsin (amo melauak)</t>
         </is>
       </c>
       <c r="F314" s="4" t="inlineStr">
@@ -10276,7 +10276,7 @@
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Red La tierra que nos une</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
@@ -10286,12 +10286,12 @@
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>{n} conjuntos de datos</t>
+          <t>WiFi gratuito: en proceso</t>
         </is>
       </c>
       <c r="E315" s="5" t="inlineStr">
         <is>
-          <t>{n} tlapoualamatl</t>
+          <t>WiFi amo iga tomin: motlalijtiga</t>
         </is>
       </c>
       <c r="F315" s="4" t="inlineStr">
@@ -10307,7 +10307,7 @@
       </c>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr">
@@ -10317,12 +10317,12 @@
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>CSV · UTF-{n}, separado por comas</t>
+          <t>Conectividad · Agencia de Transformación Digital</t>
         </is>
       </c>
       <c r="E316" s="5" t="inlineStr">
         <is>
-          <t>CSV · UTF-{n}, xeloltok iga comas</t>
+          <t>Mosaloua · Agencia de Transformación Digital</t>
         </is>
       </c>
       <c r="F316" s="4" t="inlineStr">
@@ -10338,7 +10338,7 @@
       </c>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr">
@@ -10348,12 +10348,12 @@
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>KML · una sola capa</t>
+          <t>Sitios y torres de telecomunicaciones de la red estatal (sitios REEM) que dan servicio a dependencias del Gobierno del Estado, planteles educativos, unidades de salud e instalaciones de seguridad en Morelos.</t>
         </is>
       </c>
       <c r="E317" s="5" t="inlineStr">
         <is>
-          <t>KML · san se tlapachtli</t>
+          <t>Sitios uan tepostlaketsalmej iga uejka tlanonotsalistle ipan imatlau Kaltlayekana (sitios REEM) tlen kinpaleuiaj teguichiualoyan iga Kaltlayekana, kaltlamachtiloyan, pajtiloyan uan kanin tlajpiaj ipan Morelos.</t>
         </is>
       </c>
       <c r="F317" s="4" t="inlineStr">
@@ -10369,7 +10369,7 @@
       </c>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr">
@@ -10379,12 +10379,12 @@
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Localidades · Propuesta Actual</t>
+          <t>Por seguridad de la infraestructura, la información se presenta agregada por municipio y sector. No se publica la ubicación exacta ni el nombre de los sitios.</t>
         </is>
       </c>
       <c r="E318" s="5" t="inlineStr">
         <is>
-          <t>Altepetsitsin · Tlen axan</t>
+          <t>Iga tlajpialistle, tlamachilistle monextia sepan iga altepetl uan teguitl. Amo monextia kanin melauak katej nin intogayo sitios.</t>
         </is>
       </c>
       <c r="F318" s="4" t="inlineStr">
@@ -10400,7 +10400,7 @@
       </c>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr">
@@ -10410,12 +10410,12 @@
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>{n} registros · {n} campos</t>
+          <t>Sitios de telecomunicaciones</t>
         </is>
       </c>
       <c r="E319" s="5" t="inlineStr">
         <is>
-          <t>{n} tlajkuilolli · {n} tlamachilistle</t>
+          <t>Sitios iga uejka tlanonotsalistle</t>
         </is>
       </c>
       <c r="F319" s="4" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr">
@@ -10441,12 +10441,12 @@
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Las localidades de los {n} polígonos vigentes con sus indicadores de población, vivienda, salud, educación, economía y marginación.</t>
+          <t>Municipios con sitios</t>
         </is>
       </c>
       <c r="E320" s="5" t="inlineStr">
         <is>
-          <t>Altepetsitsin tlen {n} polígono tlen axan iga itlapoual tlatlaga, kalmej, pajtilistle, temachtilistle, tomin uan iknoyotl.</t>
+          <t>Altepemej iga sitios</t>
         </is>
       </c>
       <c r="F320" s="4" t="inlineStr">
@@ -10462,7 +10462,7 @@
       </c>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr">
@@ -10472,12 +10472,12 @@
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Fuente: INEGI, Censo {n} (ITER Morelos) y Lista de Comunidades TPBV {n}</t>
+          <t>Sectores atendidos</t>
         </is>
       </c>
       <c r="E321" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: INEGI, Censo {n} (ITER Morelos) uan Lista de Comunidades TPBV {n}</t>
+          <t>Teguimej tlen kinpaleuiaj</t>
         </is>
       </c>
       <c r="F321" s="4" t="inlineStr">
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C322" s="4" t="inlineStr">
@@ -10503,12 +10503,12 @@
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Ver campos</t>
+          <t>Mayor concentración ({n} sitios)</t>
         </is>
       </c>
       <c r="E322" s="5" t="inlineStr">
         <is>
-          <t>Xikita tlen kipia</t>
+          <t>Kanin ogachi miak ({n} sitios)</t>
         </is>
       </c>
       <c r="F322" s="4" t="inlineStr">
@@ -10524,22 +10524,22 @@
       </c>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Descargar Localidades · Propuesta Actual en CSV</t>
+          <t>Sitios por municipio</t>
         </is>
       </c>
       <c r="E323" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Altepetsitsin · Tlen axan ipan CSV</t>
+          <t>Sitios iga altepetl</t>
         </is>
       </c>
       <c r="F323" s="4" t="inlineStr">
@@ -10555,22 +10555,22 @@
       </c>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Descargar Localidades · Propuesta Actual en KML</t>
+          <t>Pasa el cursor sobre un municipio para ver el desglose por sector.</t>
         </is>
       </c>
       <c r="E324" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Altepetsitsin · Tlen axan ipan KML</t>
+          <t>Xikpano tepostlapacholi ipan se altepetl iga tikitas tlen kipia iga teguitl.</t>
         </is>
       </c>
       <c r="F324" s="4" t="inlineStr">
@@ -10586,7 +10586,7 @@
       </c>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr">
@@ -10596,12 +10596,12 @@
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Polígonos · Propuesta Actual</t>
+          <t>{n} o más</t>
         </is>
       </c>
       <c r="E325" s="5" t="inlineStr">
         <is>
-          <t>Polígono · Tlen axan</t>
+          <t>{n} o ogachi</t>
         </is>
       </c>
       <c r="F325" s="4" t="inlineStr">
@@ -10617,7 +10617,7 @@
       </c>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr">
@@ -10627,12 +10627,12 @@
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Contorno de los {n} polígonos vigentes de Territorios de Paz y Buen Vivir, con número de localidades y población.</t>
+          <t>Sin sitios</t>
         </is>
       </c>
       <c r="E326" s="5" t="inlineStr">
         <is>
-          <t>Itlalxelol {n} polígono tlen axan ipan Territorios de Paz y Buen Vivir, iga keski altepetsitsin uan tlatlaga.</t>
+          <t>Amo kipia sitios</t>
         </is>
       </c>
       <c r="F326" s="4" t="inlineStr">
@@ -10648,7 +10648,7 @@
       </c>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr">
@@ -10658,12 +10658,12 @@
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>Fuente: TPBV {n}.geojson</t>
+          <t>Sitios por sector</t>
         </is>
       </c>
       <c r="E327" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: TPBV {n}.geojson</t>
+          <t>Sitios iga teguitl</t>
         </is>
       </c>
       <c r="F327" s="4" t="inlineStr">
@@ -10679,22 +10679,22 @@
       </c>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Descargar Polígonos · Propuesta Actual en CSV</t>
+          <t>Gobierno del Estado</t>
         </is>
       </c>
       <c r="E328" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Polígono · Tlen axan ipan CSV</t>
+          <t>Kaltlayekana</t>
         </is>
       </c>
       <c r="F328" s="4" t="inlineStr">
@@ -10710,22 +10710,22 @@
       </c>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>Descargar Polígonos · Propuesta Actual en KML</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="E329" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Polígono · Tlen axan ipan KML</t>
+          <t>Pajtilistle</t>
         </is>
       </c>
       <c r="F329" s="4" t="inlineStr">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr">
@@ -10751,12 +10751,12 @@
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Escuelas donde ATDEM instaló aulas de cómputo: CCT, nivel, computadoras, fecha de instalación y polígono TPBV.</t>
+          <t>Seguridad y Protección Ciudadana</t>
         </is>
       </c>
       <c r="E330" s="5" t="inlineStr">
         <is>
-          <t>Kaltlamachtiloyan kanin ATDEM kitlalij tepostlapoualli: CCT, temachtilistle, tepostlapoualmej, kemanian motlalij uan polígono TPBV.</t>
+          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga</t>
         </is>
       </c>
       <c r="F330" s="4" t="inlineStr">
@@ -10772,7 +10772,7 @@
       </c>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C331" s="4" t="inlineStr">
@@ -10782,12 +10782,12 @@
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, Proyecto Escuelas entrega Computadoras</t>
+          <t>Municipios con infraestructura</t>
         </is>
       </c>
       <c r="E331" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, Proyecto Escuelas entrega Computadoras</t>
+          <t>Altepemej iga tepostlaketsalmej</t>
         </is>
       </c>
       <c r="F331" s="4" t="inlineStr">
@@ -10803,22 +10803,22 @@
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>Descargar Aulas Tecnológicas en CSV</t>
+          <t>Sectores</t>
         </is>
       </c>
       <c r="E332" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan CSV</t>
+          <t>Teguimej</t>
         </is>
       </c>
       <c r="F332" s="4" t="inlineStr">
@@ -10834,22 +10834,22 @@
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>Descargar Aulas Tecnológicas en KML</t>
+          <t>Sitios</t>
         </is>
       </c>
       <c r="E333" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan KML</t>
+          <t>Sitios</t>
         </is>
       </c>
       <c r="F333" s="4" t="inlineStr">
@@ -10865,7 +10865,7 @@
       </c>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr">
@@ -10875,12 +10875,12 @@
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Dependencias estatales con la red Wi-Fi pública de la ATDEM: secretaría, sede, coordenadas y puntos de acceso.</t>
+          <t>Gobierno del Estado · {n}</t>
         </is>
       </c>
       <c r="E334" s="5" t="inlineStr">
         <is>
-          <t>Teguichiualoyan iga Kaltlayekana tlen kipiaj matlatl Wi-Fi tlen ATDEM: secretaría, kalle, kanin katej uan kanin mosaloua.</t>
+          <t>Kaltlayekana · {n}</t>
         </is>
       </c>
       <c r="F334" s="4" t="inlineStr">
@@ -10896,7 +10896,7 @@
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
@@ -10906,12 +10906,12 @@
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>Fuente: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+          <t>Salud · {n}</t>
         </is>
       </c>
       <c r="E335" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+          <t>Pajtilistle · {n}</t>
         </is>
       </c>
       <c r="F335" s="4" t="inlineStr">
@@ -10927,22 +10927,22 @@
       </c>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>Descargar Red La tierra que nos une en CSV</t>
+          <t>Educación · {n}</t>
         </is>
       </c>
       <c r="E336" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan CSV</t>
+          <t>Temachtilistle · {n}</t>
         </is>
       </c>
       <c r="F336" s="4" t="inlineStr">
@@ -10958,22 +10958,22 @@
       </c>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>Descargar Red La tierra que nos une en KML</t>
+          <t>Seguridad y Protección Ciudadana · {n}</t>
         </is>
       </c>
       <c r="E337" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan KML</t>
+          <t>Tlajpialistle uan Tlapaleuilistle iga Tlatlaga · {n}</t>
         </is>
       </c>
       <c r="F337" s="4" t="inlineStr">
@@ -10989,7 +10989,7 @@
       </c>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>Datos Abiertos</t>
+          <t>Infraestructura de Telecomunicaciones</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr">
@@ -10999,12 +10999,12 @@
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>Límites municipales de Morelos</t>
+          <t>Fuente: ATDEM, registro de sitios REEM. Municipio asignado con los límites municipales del INE.</t>
         </is>
       </c>
       <c r="E338" s="5" t="inlineStr">
         <is>
-          <t>Itlalxelol altepemej ipan Morelos</t>
+          <t>Kanin eua: ATDEM, sitios REEM. Altepetl motlalij iga itlalxelol altepemej tlen INE.</t>
         </is>
       </c>
       <c r="F338" s="4" t="inlineStr">
@@ -11030,12 +11030,12 @@
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>Contorno de los {n} municipios del estado, con clave geoestadística (CVEGEO) y nombre.</t>
+          <t>Territorios de Paz y Buen Vivir · Transparencia</t>
         </is>
       </c>
       <c r="E339" s="5" t="inlineStr">
         <is>
-          <t>Itlalxelol {n} altepemej, iga iclave geoestadística (CVEGEO) uan itoga.</t>
+          <t>Territorios de Paz y Buen Vivir · Tlen nochi ueli kitaskej</t>
         </is>
       </c>
       <c r="F339" s="4" t="inlineStr">
@@ -11061,12 +11061,12 @@
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>Fuente: INE, límites municipales</t>
+          <t>Descarga las bases de datos que alimentan este tablero. Cada conjunto está disponible en CSV, para abrirlo en Excel o cualquier herramienta de análisis, y en KML, para verlo en Google Earth o Google My Maps.</t>
         </is>
       </c>
       <c r="E340" s="5" t="inlineStr">
         <is>
-          <t>Kanin eua: INE, itlalxelol altepemej</t>
+          <t>Xikuiga tlapoualli tlen kitekiutia nin tablero. Nochi kipia CSV, iga tiktlapos ipan Excel o siguin programa, uan KML, iga tikitas ipan Google Earth o Google My Maps.</t>
         </is>
       </c>
       <c r="F340" s="4" t="inlineStr">
@@ -11087,17 +11087,17 @@
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>Descargar Límites municipales de Morelos en CSV</t>
+          <t>{n} conjuntos de datos</t>
         </is>
       </c>
       <c r="E341" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan CSV</t>
+          <t>{n} tlapoualamatl</t>
         </is>
       </c>
       <c r="F341" s="4" t="inlineStr">
@@ -11118,17 +11118,17 @@
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>atributo</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>Descargar Límites municipales de Morelos en KML</t>
+          <t>CSV · UTF-{n}, separado por comas</t>
         </is>
       </c>
       <c r="E342" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan KML</t>
+          <t>CSV · UTF-{n}, xeloltok iga comas</t>
         </is>
       </c>
       <c r="F342" s="4" t="inlineStr">
@@ -11154,12 +11154,12 @@
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>Los archivos se generan en tu navegador con la misma información que muestra el tablero. Para Google My Maps importa el KML en una capa nueva y usa "Aplicar estilo por columna de datos" para colorear por municipio, polígono u otro campo.</t>
+          <t>KML · una sola capa</t>
         </is>
       </c>
       <c r="E343" s="5" t="inlineStr">
         <is>
-          <t>Nin amatl mochiua ipan motepostlapoual iga nochi tlamachilistle tlen kinextia nin tablero. Iga Google My Maps, xikalaki KML ipan se yankuik tlapachtli uan xiktekiuti "Aplicar estilo por columna de datos" iga tiktlapaluis iga altepetl, polígono o siguin.</t>
+          <t>KML · san se tlapachtli</t>
         </is>
       </c>
       <c r="F343" s="4" t="inlineStr">
@@ -11175,7 +11175,7 @@
       </c>
       <c r="B344" s="4" t="inlineStr">
         <is>
-          <t>Inicio (buscador de comunidades)</t>
+          <t>Datos Abiertos</t>
         </is>
       </c>
       <c r="C344" s="4" t="inlineStr">
@@ -11185,12 +11185,12 @@
       </c>
       <c r="D344" s="4" t="inlineStr">
         <is>
-          <t>No encontramos «{d}» entre las {n} comunidades del programa. Revisa cómo está escrito o busca por municipio.</t>
+          <t>Localidades · Propuesta Actual</t>
         </is>
       </c>
       <c r="E344" s="5" t="inlineStr">
         <is>
-          <t>Amo otikajsike «{d}» ipan {n} altepetsitsin tlen nin tlapaleuilistle. Xiktlachili kenin otiktlajkuilo o xiktemo iga altepetl.</t>
+          <t>Altepetsitsin · Tlen axan</t>
         </is>
       </c>
       <c r="F344" s="4" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="B345" s="4" t="inlineStr">
         <is>
-          <t>Inicio (buscador de comunidades)</t>
+          <t>Datos Abiertos</t>
         </is>
       </c>
       <c r="C345" s="4" t="inlineStr">
@@ -11216,12 +11216,12 @@
       </c>
       <c r="D345" s="4" t="inlineStr">
         <is>
-          <t>{d} tiene {n} comunidad en el programa.</t>
+          <t>{n} registros · {n} campos</t>
         </is>
       </c>
       <c r="E345" s="5" t="inlineStr">
         <is>
-          <t>{d} kipia {n} altepetsin ipan nin tlapaleuilistle.</t>
+          <t>{n} tlajkuilolli · {n} tlamachilistle</t>
         </is>
       </c>
       <c r="F345" s="4" t="inlineStr">
@@ -11237,7 +11237,7 @@
       </c>
       <c r="B346" s="4" t="inlineStr">
         <is>
-          <t>Inicio (buscador de comunidades)</t>
+          <t>Datos Abiertos</t>
         </is>
       </c>
       <c r="C346" s="4" t="inlineStr">
@@ -11247,12 +11247,12 @@
       </c>
       <c r="D346" s="4" t="inlineStr">
         <is>
-          <t>Y {n} comunidad más. Escribe más letras para afinar la búsqueda.</t>
+          <t>Las localidades de los {n} polígonos vigentes con sus indicadores de población, vivienda, salud, educación, economía y marginación.</t>
         </is>
       </c>
       <c r="E346" s="5" t="inlineStr">
         <is>
-          <t>Uan ogachi {n} altepetsin. Xiktlajkuilo ogachi tlajkuilolli iga tiktemos kuale.</t>
+          <t>Altepetsitsin tlen {n} polígono tlen axan iga itlapoual tlatlaga, kalmej, pajtilistle, temachtilistle, tomin uan iknoyotl.</t>
         </is>
       </c>
       <c r="F346" s="4" t="inlineStr">
@@ -11268,33 +11268,994 @@
       </c>
       <c r="B347" s="4" t="inlineStr">
         <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C347" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D347" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: INEGI, Censo {n} (ITER Morelos) y Lista de Comunidades TPBV {n}</t>
+        </is>
+      </c>
+      <c r="E347" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: INEGI, Censo {n} (ITER Morelos) uan Lista de Comunidades TPBV {n}</t>
+        </is>
+      </c>
+      <c r="F347" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G347" s="4" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="4" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C348" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D348" s="4" t="inlineStr">
+        <is>
+          <t>Ver campos</t>
+        </is>
+      </c>
+      <c r="E348" s="5" t="inlineStr">
+        <is>
+          <t>Xikita tlen kipia</t>
+        </is>
+      </c>
+      <c r="F348" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G348" s="4" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="4" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C349" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D349" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Localidades · Propuesta Actual en CSV</t>
+        </is>
+      </c>
+      <c r="E349" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Altepetsitsin · Tlen axan ipan CSV</t>
+        </is>
+      </c>
+      <c r="F349" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G349" s="4" t="n"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="4" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C350" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D350" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Localidades · Propuesta Actual en KML</t>
+        </is>
+      </c>
+      <c r="E350" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Altepetsitsin · Tlen axan ipan KML</t>
+        </is>
+      </c>
+      <c r="F350" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G350" s="4" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C351" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D351" s="4" t="inlineStr">
+        <is>
+          <t>Polígonos · Propuesta Actual</t>
+        </is>
+      </c>
+      <c r="E351" s="5" t="inlineStr">
+        <is>
+          <t>Polígono · Tlen axan</t>
+        </is>
+      </c>
+      <c r="F351" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G351" s="4" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="4" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C352" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D352" s="4" t="inlineStr">
+        <is>
+          <t>Contorno de los {n} polígonos vigentes de Territorios de Paz y Buen Vivir, con número de localidades y población.</t>
+        </is>
+      </c>
+      <c r="E352" s="5" t="inlineStr">
+        <is>
+          <t>Itlalxelol {n} polígono tlen axan ipan Territorios de Paz y Buen Vivir, iga keski altepetsitsin uan tlatlaga.</t>
+        </is>
+      </c>
+      <c r="F352" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G352" s="4" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="4" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C353" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D353" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: TPBV {n}.geojson</t>
+        </is>
+      </c>
+      <c r="E353" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: TPBV {n}.geojson</t>
+        </is>
+      </c>
+      <c r="F353" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G353" s="4" t="n"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="4" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C354" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D354" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Polígonos · Propuesta Actual en CSV</t>
+        </is>
+      </c>
+      <c r="E354" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Polígono · Tlen axan ipan CSV</t>
+        </is>
+      </c>
+      <c r="F354" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G354" s="4" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="4" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C355" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D355" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Polígonos · Propuesta Actual en KML</t>
+        </is>
+      </c>
+      <c r="E355" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Polígono · Tlen axan ipan KML</t>
+        </is>
+      </c>
+      <c r="F355" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G355" s="4" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C356" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D356" s="4" t="inlineStr">
+        <is>
+          <t>Escuelas donde ATDEM instaló aulas de cómputo: CCT, nivel, computadoras, fecha de instalación y polígono TPBV.</t>
+        </is>
+      </c>
+      <c r="E356" s="5" t="inlineStr">
+        <is>
+          <t>Kaltlamachtiloyan kanin ATDEM kitlalij tepostlapoualli: CCT, temachtilistle, tepostlapoualmej, kemanian motlalij uan polígono TPBV.</t>
+        </is>
+      </c>
+      <c r="F356" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G356" s="4" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="4" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C357" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D357" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: ATDEM, Proyecto Escuelas entrega Computadoras</t>
+        </is>
+      </c>
+      <c r="E357" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: ATDEM, Proyecto Escuelas entrega Computadoras</t>
+        </is>
+      </c>
+      <c r="F357" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G357" s="4" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C358" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D358" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Aulas Tecnológicas en CSV</t>
+        </is>
+      </c>
+      <c r="E358" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan CSV</t>
+        </is>
+      </c>
+      <c r="F358" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G358" s="4" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Aulas Tecnológicas en KML</t>
+        </is>
+      </c>
+      <c r="E359" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Tlamachtiloyan iga tepostlapoualli ipan KML</t>
+        </is>
+      </c>
+      <c r="F359" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G359" s="4" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C360" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D360" s="4" t="inlineStr">
+        <is>
+          <t>Dependencias estatales con la red Wi-Fi pública de la ATDEM: secretaría, sede, coordenadas y puntos de acceso.</t>
+        </is>
+      </c>
+      <c r="E360" s="5" t="inlineStr">
+        <is>
+          <t>Teguichiualoyan iga Kaltlayekana tlen kipiaj matlatl Wi-Fi tlen ATDEM: secretaría, kalle, kanin katej uan kanin mosaloua.</t>
+        </is>
+      </c>
+      <c r="F360" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G360" s="4" t="n"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="4" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C361" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D361" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+        </is>
+      </c>
+      <c r="E361" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: ATDEM, Agentes_dependencias La Tierra Que Nos Une</t>
+        </is>
+      </c>
+      <c r="F361" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G361" s="4" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C362" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D362" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Red La tierra que nos une en CSV</t>
+        </is>
+      </c>
+      <c r="E362" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan CSV</t>
+        </is>
+      </c>
+      <c r="F362" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G362" s="4" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="4" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C363" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D363" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Red La tierra que nos une en KML</t>
+        </is>
+      </c>
+      <c r="E363" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Matlatl Nin tlale tech sepaneloa ipan KML</t>
+        </is>
+      </c>
+      <c r="F363" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G363" s="4" t="n"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="4" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C364" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D364" s="4" t="inlineStr">
+        <is>
+          <t>Red La tierra que nos une · Comunidades</t>
+        </is>
+      </c>
+      <c r="E364" s="5" t="inlineStr">
+        <is>
+          <t>Matlatl Nin tlale tech sepaneloa · Altepetsitsin</t>
+        </is>
+      </c>
+      <c r="F364" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G364" s="4" t="n"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="4" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C365" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D365" s="4" t="inlineStr">
+        <is>
+          <t>Comunidades con WiFi gratuito de la ATDEM instalado o en proceso: localidad, municipio, coordenadas, estatus y polígono TPBV.</t>
+        </is>
+      </c>
+      <c r="E365" s="5" t="inlineStr">
+        <is>
+          <t>Altepetsitsin iga WiFi amo iga tomin tlen ATDEM tlen motlalij o motlalijtiga: altepetsin, altepetl, kanin katej, kenin katej uan polígono TPBV.</t>
+        </is>
+      </c>
+      <c r="F365" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G365" s="4" t="n"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="4" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C366" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D366" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: ATDEM, registro de instalaciones en comunidades</t>
+        </is>
+      </c>
+      <c r="E366" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: ATDEM, itlajkuilol tlen motlalij ipan altepetsitsin</t>
+        </is>
+      </c>
+      <c r="F366" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G366" s="4" t="n"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="4" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C367" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D367" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Red La tierra que nos une · Comunidades en CSV</t>
+        </is>
+      </c>
+      <c r="E367" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Matlatl Nin tlale tech sepaneloa · Altepetsitsin ipan CSV</t>
+        </is>
+      </c>
+      <c r="F367" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G367" s="4" t="n"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="4" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C368" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D368" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Red La tierra que nos une · Comunidades en KML</t>
+        </is>
+      </c>
+      <c r="E368" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Matlatl Nin tlale tech sepaneloa · Altepetsitsin ipan KML</t>
+        </is>
+      </c>
+      <c r="F368" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G368" s="4" t="n"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="4" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C369" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D369" s="4" t="inlineStr">
+        <is>
+          <t>Límites municipales de Morelos</t>
+        </is>
+      </c>
+      <c r="E369" s="5" t="inlineStr">
+        <is>
+          <t>Itlalxelol altepemej ipan Morelos</t>
+        </is>
+      </c>
+      <c r="F369" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G369" s="4" t="n"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="4" t="n">
+        <v>369</v>
+      </c>
+      <c r="B370" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C370" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D370" s="4" t="inlineStr">
+        <is>
+          <t>Contorno de los {n} municipios del estado, con clave geoestadística (CVEGEO) y nombre.</t>
+        </is>
+      </c>
+      <c r="E370" s="5" t="inlineStr">
+        <is>
+          <t>Itlalxelol {n} altepemej, iga iclave geoestadística (CVEGEO) uan itoga.</t>
+        </is>
+      </c>
+      <c r="F370" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G370" s="4" t="n"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="4" t="n">
+        <v>370</v>
+      </c>
+      <c r="B371" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C371" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D371" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: INE, límites municipales</t>
+        </is>
+      </c>
+      <c r="E371" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: INE, itlalxelol altepemej</t>
+        </is>
+      </c>
+      <c r="F371" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G371" s="4" t="n"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="4" t="n">
+        <v>371</v>
+      </c>
+      <c r="B372" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C372" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D372" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Límites municipales de Morelos en CSV</t>
+        </is>
+      </c>
+      <c r="E372" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan CSV</t>
+        </is>
+      </c>
+      <c r="F372" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G372" s="4" t="n"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="4" t="n">
+        <v>372</v>
+      </c>
+      <c r="B373" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C373" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D373" s="4" t="inlineStr">
+        <is>
+          <t>Descargar Límites municipales de Morelos en KML</t>
+        </is>
+      </c>
+      <c r="E373" s="5" t="inlineStr">
+        <is>
+          <t>Xikuiga Itlalxelol altepemej ipan Morelos ipan KML</t>
+        </is>
+      </c>
+      <c r="F373" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G373" s="4" t="n"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="4" t="n">
+        <v>373</v>
+      </c>
+      <c r="B374" s="4" t="inlineStr">
+        <is>
+          <t>Datos Abiertos</t>
+        </is>
+      </c>
+      <c r="C374" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D374" s="4" t="inlineStr">
+        <is>
+          <t>Los archivos se generan en tu navegador con la misma información que muestra el tablero. Para Google My Maps importa el KML en una capa nueva y usa "Aplicar estilo por columna de datos" para colorear por municipio, polígono u otro campo.</t>
+        </is>
+      </c>
+      <c r="E374" s="5" t="inlineStr">
+        <is>
+          <t>Nin amatl mochiua ipan motepostlapoual iga nochi tlamachilistle tlen kinextia nin tablero. Iga Google My Maps, xikalaki KML ipan se yankuik tlapachtli uan xiktekiuti "Aplicar estilo por columna de datos" iga tiktlapaluis iga altepetl, polígono o siguin.</t>
+        </is>
+      </c>
+      <c r="F374" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G374" s="4" t="n"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="4" t="n">
+        <v>374</v>
+      </c>
+      <c r="B375" s="4" t="inlineStr">
+        <is>
+          <t>Inicio (buscador de comunidades)</t>
+        </is>
+      </c>
+      <c r="C375" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D375" s="4" t="inlineStr">
+        <is>
+          <t>No encontramos «{d}» entre las {n} comunidades del programa. Revisa cómo está escrito o busca por municipio.</t>
+        </is>
+      </c>
+      <c r="E375" s="5" t="inlineStr">
+        <is>
+          <t>Amo otikajsike «{d}» ipan {n} altepetsitsin tlen nin tlapaleuilistle. Xiktlachili kenin otiktlajkuilo o xiktemo iga altepetl.</t>
+        </is>
+      </c>
+      <c r="F375" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G375" s="4" t="n"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="4" t="n">
+        <v>375</v>
+      </c>
+      <c r="B376" s="4" t="inlineStr">
+        <is>
+          <t>Inicio (buscador de comunidades)</t>
+        </is>
+      </c>
+      <c r="C376" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D376" s="4" t="inlineStr">
+        <is>
+          <t>{d} tiene {n} comunidad en el programa.</t>
+        </is>
+      </c>
+      <c r="E376" s="5" t="inlineStr">
+        <is>
+          <t>{d} kipia {n} altepetsin ipan nin tlapaleuilistle.</t>
+        </is>
+      </c>
+      <c r="F376" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G376" s="4" t="n"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="4" t="n">
+        <v>376</v>
+      </c>
+      <c r="B377" s="4" t="inlineStr">
+        <is>
+          <t>Inicio (buscador de comunidades)</t>
+        </is>
+      </c>
+      <c r="C377" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D377" s="4" t="inlineStr">
+        <is>
+          <t>Y {n} comunidad más. Escribe más letras para afinar la búsqueda.</t>
+        </is>
+      </c>
+      <c r="E377" s="5" t="inlineStr">
+        <is>
+          <t>Uan ogachi {n} altepetsin. Xiktlajkuilo ogachi tlajkuilolli iga tiktemos kuale.</t>
+        </is>
+      </c>
+      <c r="F377" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G377" s="4" t="n"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="4" t="n">
+        <v>377</v>
+      </c>
+      <c r="B378" s="4" t="inlineStr">
+        <is>
           <t>Encabezado y menú</t>
         </is>
       </c>
-      <c r="C347" s="4" t="inlineStr">
+      <c r="C378" s="4" t="inlineStr">
         <is>
           <t>atributo</t>
         </is>
       </c>
-      <c r="D347" s="4" t="inlineStr">
+      <c r="D378" s="4" t="inlineStr">
         <is>
           <t>Territorios de Paz y Buen Vivir · Gobierno de Morelos</t>
         </is>
       </c>
-      <c r="E347" s="5" t="inlineStr">
+      <c r="E378" s="5" t="inlineStr">
         <is>
           <t>Territorios de Paz y Buen Vivir · Kaltlayekana ipan Morelos</t>
         </is>
       </c>
-      <c r="F347" s="4" t="inlineStr">
-        <is>
-          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
-        </is>
-      </c>
-      <c r="G347" s="4" t="n"/>
+      <c r="F378" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G378" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G347"/>
+  <autoFilter ref="A1:G378"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: Datos Abiertos nombra Localidades y Poligonos TPBV 2026 en lugar de Propuesta Actual
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traducciones/Traduccion_nahuatl_tablero.xlsx
+++ b/traducciones/Traduccion_nahuatl_tablero.xlsx
@@ -11185,12 +11185,12 @@
       </c>
       <c r="D344" s="4" t="inlineStr">
         <is>
-          <t>Localidades · Propuesta Actual</t>
+          <t>Localidades TPBV {n}</t>
         </is>
       </c>
       <c r="E344" s="5" t="inlineStr">
         <is>
-          <t>Altepetsitsin · Tlen axan</t>
+          <t>Altepetsitsin TPBV {n}</t>
         </is>
       </c>
       <c r="F344" s="4" t="inlineStr">
@@ -11340,12 +11340,12 @@
       </c>
       <c r="D349" s="4" t="inlineStr">
         <is>
-          <t>Descargar Localidades · Propuesta Actual en CSV</t>
+          <t>Descargar Localidades TPBV {n} en CSV</t>
         </is>
       </c>
       <c r="E349" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Altepetsitsin · Tlen axan ipan CSV</t>
+          <t>Xikuiga Altepetsitsin TPBV {n} ipan CSV</t>
         </is>
       </c>
       <c r="F349" s="4" t="inlineStr">
@@ -11371,12 +11371,12 @@
       </c>
       <c r="D350" s="4" t="inlineStr">
         <is>
-          <t>Descargar Localidades · Propuesta Actual en KML</t>
+          <t>Descargar Localidades TPBV {n} en KML</t>
         </is>
       </c>
       <c r="E350" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Altepetsitsin · Tlen axan ipan KML</t>
+          <t>Xikuiga Altepetsitsin TPBV {n} ipan KML</t>
         </is>
       </c>
       <c r="F350" s="4" t="inlineStr">
@@ -11402,12 +11402,12 @@
       </c>
       <c r="D351" s="4" t="inlineStr">
         <is>
-          <t>Polígonos · Propuesta Actual</t>
+          <t>Polígonos TPBV {n}</t>
         </is>
       </c>
       <c r="E351" s="5" t="inlineStr">
         <is>
-          <t>Polígono · Tlen axan</t>
+          <t>Polígono TPBV {n}</t>
         </is>
       </c>
       <c r="F351" s="4" t="inlineStr">
@@ -11495,12 +11495,12 @@
       </c>
       <c r="D354" s="4" t="inlineStr">
         <is>
-          <t>Descargar Polígonos · Propuesta Actual en CSV</t>
+          <t>Descargar Polígonos TPBV {n} en CSV</t>
         </is>
       </c>
       <c r="E354" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Polígono · Tlen axan ipan CSV</t>
+          <t>Xikuiga Polígono TPBV {n} ipan CSV</t>
         </is>
       </c>
       <c r="F354" s="4" t="inlineStr">
@@ -11526,12 +11526,12 @@
       </c>
       <c r="D355" s="4" t="inlineStr">
         <is>
-          <t>Descargar Polígonos · Propuesta Actual en KML</t>
+          <t>Descargar Polígonos TPBV {n} en KML</t>
         </is>
       </c>
       <c r="E355" s="5" t="inlineStr">
         <is>
-          <t>Xikuiga Polígono · Tlen axan ipan KML</t>
+          <t>Xikuiga Polígono TPBV {n} ipan KML</t>
         </is>
       </c>
       <c r="F355" s="4" t="inlineStr">

</xml_diff>

<commit_message>
feat: ajustes del Morelos Design System (accesibilidad, ancho, colores, tarjetas y ruta)
- Ancho maximo de contenido 1440 px y colores de estado del DS
- Contraste AA en el encabezado; descargas de Datos Abiertos con contorno
- accesibilidad.js: aviso de pestana nueva e iconos ocultos a lectores
- Tarjetas de Inicio clicables completas, enlaces subrayados
- Ruta de navegacion en Analisis (analisis_migas.js)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traducciones/Traduccion_nahuatl_tablero.xlsx
+++ b/traducciones/Traduccion_nahuatl_tablero.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G378"/>
+  <dimension ref="A1:G381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12253,6 +12253,111 @@
         </is>
       </c>
       <c r="G378" s="4" t="n"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="4" t="n">
+        <v>378</v>
+      </c>
+      <c r="B379" s="4" t="inlineStr">
+        <is>
+          <t>General (lectores de pantalla)</t>
+        </is>
+      </c>
+      <c r="C379" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D379" s="4" t="inlineStr">
+        <is>
+          <t>(se abre en una pestaña nueva)</t>
+        </is>
+      </c>
+      <c r="E379" s="5" t="inlineStr">
+        <is>
+          <t>(motlapoua ipan okse amatl)</t>
+        </is>
+      </c>
+      <c r="F379" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G379" s="4" t="inlineStr">
+        <is>
+          <t>Aviso para lectores de pantalla en enlaces que abren pestaña nueva</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="B380" s="4" t="inlineStr">
+        <is>
+          <t>Análisis Demográfico</t>
+        </is>
+      </c>
+      <c r="C380" s="4" t="inlineStr">
+        <is>
+          <t>atributo</t>
+        </is>
+      </c>
+      <c r="D380" s="4" t="inlineStr">
+        <is>
+          <t>Ruta de navegación</t>
+        </is>
+      </c>
+      <c r="E380" s="5" t="inlineStr">
+        <is>
+          <t>Ojtle kanin tinemi</t>
+        </is>
+      </c>
+      <c r="F380" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G380" s="4" t="inlineStr">
+        <is>
+          <t>Ruta (breadcrumbs) de Análisis, para lectores de pantalla</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="4" t="n">
+        <v>380</v>
+      </c>
+      <c r="B381" s="4" t="inlineStr">
+        <is>
+          <t>Análisis Demográfico</t>
+        </is>
+      </c>
+      <c r="C381" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D381" s="4" t="inlineStr">
+        <is>
+          <t>Comparación de {n} polígonos</t>
+        </is>
+      </c>
+      <c r="E381" s="5" t="inlineStr">
+        <is>
+          <t>Tikinneneuilia {n} polígono</t>
+        </is>
+      </c>
+      <c r="F381" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G381" s="4" t="inlineStr">
+        <is>
+          <t>Último nivel de la ruta al comparar polígonos</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G378"/>

</xml_diff>

<commit_message>
feat: Red solo con WiFi en comunidades en TPBV; pagina nueva de Conectividad
- RED_MOSTRAR_OFICINAS = false: el tablero TPBV oculta cifras, mapa, lista
  y conjunto de Datos Abiertos de las oficinas de gobierno
- conectividad.html (Telecomunicaciones + Red) con comun.js compartido;
  embed_dashboard.py procesa las dos paginas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traducciones/Traduccion_nahuatl_tablero.xlsx
+++ b/traducciones/Traduccion_nahuatl_tablero.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G381"/>
+  <dimension ref="A1:G383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12356,6 +12356,76 @@
       <c r="G381" s="4" t="inlineStr">
         <is>
           <t>Último nivel de la ruta al comparar polígonos</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="4" t="n">
+        <v>381</v>
+      </c>
+      <c r="B382" s="4" t="inlineStr">
+        <is>
+          <t>Inicio</t>
+        </is>
+      </c>
+      <c r="C382" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D382" s="4" t="inlineStr">
+        <is>
+          <t>Mapa del WiFi gratuito de la ATDEM en comunidades: dónde ya está instalado y dónde está en proceso.</t>
+        </is>
+      </c>
+      <c r="E382" s="5" t="inlineStr">
+        <is>
+          <t>Itlalamauj WiFi amo iga tomin tlen ATDEM ipan altepetsitsin: kanin ya motlalij uan kanin motlalijtiga.</t>
+        </is>
+      </c>
+      <c r="F382" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G382" s="4" t="inlineStr">
+        <is>
+          <t>Tarjeta de Red en Inicio (sin oficinas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="4" t="n">
+        <v>382</v>
+      </c>
+      <c r="B383" s="4" t="inlineStr">
+        <is>
+          <t>Red La tierra que nos une</t>
+        </is>
+      </c>
+      <c r="C383" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="D383" s="4" t="inlineStr">
+        <is>
+          <t>Fuente: ATDEM, registro de instalaciones de WiFi gratuito en comunidades.</t>
+        </is>
+      </c>
+      <c r="E383" s="5" t="inlineStr">
+        <is>
+          <t>Kanin eua: ATDEM, itlajkuilol tlen WiFi amo iga tomin tlen motlalij ipan altepetsitsin.</t>
+        </is>
+      </c>
+      <c r="F383" s="4" t="inlineStr">
+        <is>
+          <t>Borrador automático, ajustado a Hueyapan (revisar)</t>
+        </is>
+      </c>
+      <c r="G383" s="4" t="inlineStr">
+        <is>
+          <t>Fuente de Red (sin oficinas)</t>
         </is>
       </c>
     </row>

</xml_diff>